<commit_message>
Add quarterly employee plan tracking
Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sales_plan_company_filled.xlsx
+++ b/sales_plan_company_filled.xlsx
@@ -8,18 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Сделки" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Сводка по компании" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Сводка по сотрудникам" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Источники" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Справочники" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Дашборд" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Сводка по сотрудникам" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Источники" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Справочники" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Дашборд" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сделки'!$A$1:$N$500</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сводка по компании'!$A$3:$N$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Сводка по сотрудникам'!$A$3:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Источники'!$A$1:$D$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Справочники'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сводка по сотрудникам'!$A$4:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники'!$A$1:$E$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Справочники'!$A$1:$N$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -109,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -130,22 +128,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -265,14 +260,64 @@
     <author>Cursor</author>
   </authors>
   <commentList>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Суммы из индивидуальных планов сотрудников. По уточнению это прогноз/пайплайн, не целевой план.</t>
+      </text>
+    </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Вероятность оставлена как справочный признак для ясности, без дополнительных расчетов.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Cursor</author>
+  </authors>
+  <commentList>
+    <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>Отклонение = факт - план. В таблице используются только суммы план и факт.</t>
+        <t>Если выбран конкретный квартал — план за квартал. Если выбрано Все — годовой план как 4 квартала.</t>
+      </text>
+    </comment>
+    <comment ref="D4" authorId="0" shapeId="0">
+      <text>
+        <t>Сумма из листа Сделки; по уточнению это прогноз/пайплайн.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Cursor</author>
+  </authors>
+  <commentList>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Настоящий план сотрудника на квартал. Суммы из листа Сделки считаются прогнозом/пайплайном.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Cursor</author>
+  </authors>
+  <commentList>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>Прогноз — это суммы из листа Сделки.</t>
       </text>
     </comment>
   </commentList>
@@ -290,11 +335,11 @@
     <tableColumn id="5" name="Подразделение"/>
     <tableColumn id="6" name="Заказчик"/>
     <tableColumn id="7" name="Вид услуги"/>
-    <tableColumn id="8" name="План"/>
+    <tableColumn id="8" name="Прогноз"/>
     <tableColumn id="9" name="Факт"/>
     <tableColumn id="10" name="Статус"/>
     <tableColumn id="11" name="Вероятность"/>
-    <tableColumn id="12" name="Отклонение"/>
+    <tableColumn id="12" name="Отклонение факт-прогноз"/>
     <tableColumn id="13" name="Комментарий"/>
     <tableColumn id="14" name="Дата обновления"/>
   </tableColumns>
@@ -605,7 +650,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="36" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
@@ -648,7 +693,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>План</t>
+          <t>Прогноз</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -668,7 +713,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Отклонение</t>
+          <t>Отклонение факт-прогноз</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
@@ -738,7 +783,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="3">
@@ -797,7 +842,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="4">
@@ -856,7 +901,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="5">
@@ -915,7 +960,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="6">
@@ -974,7 +1019,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="7">
@@ -1033,7 +1078,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="8">
@@ -1092,7 +1137,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr"/>
       <c r="N8" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="9">
@@ -1151,7 +1196,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="10">
@@ -1210,7 +1255,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="11">
@@ -1269,7 +1314,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="12">
@@ -1328,7 +1373,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr"/>
       <c r="N12" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="13">
@@ -1387,7 +1432,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="14">
@@ -1446,7 +1491,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="15">
@@ -1505,7 +1550,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr"/>
       <c r="N15" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="16">
@@ -1564,7 +1609,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1668,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr"/>
       <c r="N17" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="18">
@@ -1682,7 +1727,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="19">
@@ -1741,7 +1786,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr"/>
       <c r="N19" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="20">
@@ -1800,7 +1845,7 @@
       </c>
       <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="21">
@@ -1859,7 +1904,7 @@
       </c>
       <c r="M21" s="4" t="inlineStr"/>
       <c r="N21" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="22">
@@ -1918,7 +1963,7 @@
       </c>
       <c r="M22" s="4" t="inlineStr"/>
       <c r="N22" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="23">
@@ -1977,7 +2022,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr"/>
       <c r="N23" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="24">
@@ -2036,7 +2081,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr"/>
       <c r="N24" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="25">
@@ -2095,7 +2140,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr"/>
       <c r="N25" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="26">
@@ -2154,7 +2199,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr"/>
       <c r="N26" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="27">
@@ -2213,7 +2258,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr"/>
       <c r="N27" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="28">
@@ -2272,7 +2317,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr"/>
       <c r="N28" s="6" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="29">
@@ -12681,15 +12726,18 @@
       <formula>$J2="Отменена"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочники!$G$2:$G$5</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочники!$E$2:$E$13</formula1>
     </dataValidation>
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Справочники!$K$2:$K$7</formula1>
+    </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Справочники!$I$2:$I$3</formula1>
+      <formula1>=Справочники!$I$2:$I$4</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Справочники!$A$2:$A$6</formula1>
@@ -12715,832 +12763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Сводка по компании: план и факт по видам услуг и месяцам, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Вид услуги</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Январь</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Февраль</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Март</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Апрель</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t>Май</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>Июнь</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>Июль</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>Август</t>
-        </is>
-      </c>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>Сентябрь</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr">
-        <is>
-          <t>Октябрь</t>
-        </is>
-      </c>
-      <c r="M3" s="1" t="inlineStr">
-        <is>
-          <t>Ноябрь</t>
-        </is>
-      </c>
-      <c r="N3" s="1" t="inlineStr">
-        <is>
-          <t>Декабрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>SaaS</t>
-        </is>
-      </c>
-      <c r="C4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B4,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>On-Premise</t>
-        </is>
-      </c>
-      <c r="C5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B5,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Услуги</t>
-        </is>
-      </c>
-      <c r="C6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B6,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Доп. план</t>
-        </is>
-      </c>
-      <c r="C7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B7,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Up-Sale</t>
-        </is>
-      </c>
-      <c r="C8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N8" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$G:$G,$B8,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>SaaS</t>
-        </is>
-      </c>
-      <c r="C9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N9" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B9,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>On-Premise</t>
-        </is>
-      </c>
-      <c r="C10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N10" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B10,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Услуги</t>
-        </is>
-      </c>
-      <c r="C11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B11,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Доп. план</t>
-        </is>
-      </c>
-      <c r="C12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B12,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Up-Sale</t>
-        </is>
-      </c>
-      <c r="C13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,C$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="D13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,D$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="E13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,E$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="F13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,F$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="G13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,G$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="H13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,H$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="I13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,I$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="J13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,J$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="K13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,K$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="L13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,L$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="M13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,M$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$G:$G,$B13,Сделки!$C:$C,N$3,Сделки!$A:$A,2026)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Итого план</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="9">
-        <f>SUM(C4:C8)</f>
-        <v/>
-      </c>
-      <c r="D14" s="9">
-        <f>SUM(D4:D8)</f>
-        <v/>
-      </c>
-      <c r="E14" s="9">
-        <f>SUM(E4:E8)</f>
-        <v/>
-      </c>
-      <c r="F14" s="9">
-        <f>SUM(F4:F8)</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
-        <f>SUM(G4:G8)</f>
-        <v/>
-      </c>
-      <c r="H14" s="9">
-        <f>SUM(H4:H8)</f>
-        <v/>
-      </c>
-      <c r="I14" s="9">
-        <f>SUM(I4:I8)</f>
-        <v/>
-      </c>
-      <c r="J14" s="9">
-        <f>SUM(J4:J8)</f>
-        <v/>
-      </c>
-      <c r="K14" s="9">
-        <f>SUM(K4:K8)</f>
-        <v/>
-      </c>
-      <c r="L14" s="9">
-        <f>SUM(L4:L8)</f>
-        <v/>
-      </c>
-      <c r="M14" s="9">
-        <f>SUM(M4:M8)</f>
-        <v/>
-      </c>
-      <c r="N14" s="9">
-        <f>SUM(N4:N8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Итого факт</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="9">
-        <f>SUM(C9:C13)</f>
-        <v/>
-      </c>
-      <c r="D15" s="9">
-        <f>SUM(D9:D13)</f>
-        <v/>
-      </c>
-      <c r="E15" s="9">
-        <f>SUM(E9:E13)</f>
-        <v/>
-      </c>
-      <c r="F15" s="9">
-        <f>SUM(F9:F13)</f>
-        <v/>
-      </c>
-      <c r="G15" s="9">
-        <f>SUM(G9:G13)</f>
-        <v/>
-      </c>
-      <c r="H15" s="9">
-        <f>SUM(H9:H13)</f>
-        <v/>
-      </c>
-      <c r="I15" s="9">
-        <f>SUM(I9:I13)</f>
-        <v/>
-      </c>
-      <c r="J15" s="9">
-        <f>SUM(J9:J13)</f>
-        <v/>
-      </c>
-      <c r="K15" s="9">
-        <f>SUM(K9:K13)</f>
-        <v/>
-      </c>
-      <c r="L15" s="9">
-        <f>SUM(L9:L13)</f>
-        <v/>
-      </c>
-      <c r="M15" s="9">
-        <f>SUM(M9:M13)</f>
-        <v/>
-      </c>
-      <c r="N15" s="9">
-        <f>SUM(N9:N13)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:N15"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13553,6 +12776,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13562,106 +12787,84 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Фильтр по кварталу</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Все</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Сотрудник</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Подразделение</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>План</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Квартальный план</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Прогноз</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Факт</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Отклонение</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>Выполнение, %</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Отклонение факт-план</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Выполнение факта, %</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Выполнение прогноза, %</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Сделок всего</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>Завершено</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="K4" s="1" t="inlineStr">
         <is>
           <t>В работе</t>
         </is>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="L4" s="1" t="inlineStr">
         <is>
           <t>Обсуждение/риски</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Петриченко Мария</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="C4" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A4)</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A4)</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>D4-C4</f>
-        <v/>
-      </c>
-      <c r="F4" s="10">
-        <f>IFERROR(D4/C4,0)</f>
-        <v/>
-      </c>
-      <c r="G4" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A4)</f>
-        <v/>
-      </c>
-      <c r="H4" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A4,Сделки!$J:$J,"Завершена")</f>
-        <v/>
-      </c>
-      <c r="I4" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A4,Сделки!$J:$J,"Планируется")</f>
-        <v/>
-      </c>
-      <c r="J4" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A4,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$D:$D,$A4,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$D:$D,$A4,Сделки!$J:$J,"Бюджет под риском")</f>
-        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Журавлев Иван</t>
+          <t>Петриченко Мария</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -13670,131 +12873,1156 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A5)</f>
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A5)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A5))</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A5)</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*Сделки!$H$2:$H$500)</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>D5-C5</f>
-        <v/>
-      </c>
-      <c r="F5" s="10">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>E5-C5</f>
+        <v/>
+      </c>
+      <c r="G5" s="9">
+        <f>IFERROR(E5/C5,0)</f>
+        <v/>
+      </c>
+      <c r="H5" s="9">
         <f>IFERROR(D5/C5,0)</f>
         <v/>
       </c>
-      <c r="G5" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A5,Сделки!$J:$J,"Завершена")</f>
-        <v/>
-      </c>
       <c r="I5" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A5,Сделки!$J:$J,"Планируется")</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="J5" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A5,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$D:$D,$A5,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$D:$D,$A5,Сделки!$J:$J,"Бюджет под риском")</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K5" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L5" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Шатнюк Дарья</t>
+          <t>Журавлев Иван</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C6" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A6)</f>
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A6)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A6))</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A6)</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*Сделки!$H$2:$H$500)</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>D6-C6</f>
-        <v/>
-      </c>
-      <c r="F6" s="10">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>E6-C6</f>
+        <v/>
+      </c>
+      <c r="G6" s="9">
+        <f>IFERROR(E6/C6,0)</f>
+        <v/>
+      </c>
+      <c r="H6" s="9">
         <f>IFERROR(D6/C6,0)</f>
         <v/>
       </c>
-      <c r="G6" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A6,Сделки!$J:$J,"Завершена")</f>
-        <v/>
-      </c>
       <c r="I6" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A6,Сделки!$J:$J,"Планируется")</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
         <v/>
       </c>
       <c r="J6" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A6,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$D:$D,$A6,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$D:$D,$A6,Сделки!$J:$J,"Бюджет под риском")</f>
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K6" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L6" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>Шатнюк Дарья</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="C7" s="5">
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A7)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A7))</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>E7-C7</f>
+        <v/>
+      </c>
+      <c r="G7" s="9">
+        <f>IFERROR(E7/C7,0)</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>IFERROR(D7/C7,0)</f>
+        <v/>
+      </c>
+      <c r="I7" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="J7" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K7" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L7" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>Смирнов Дмитрий</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>BI</t>
         </is>
       </c>
-      <c r="C7" s="5">
-        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A7)</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A7)</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>D7-C7</f>
-        <v/>
-      </c>
-      <c r="F7" s="10">
-        <f>IFERROR(D7/C7,0)</f>
-        <v/>
-      </c>
-      <c r="G7" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A7,Сделки!$J:$J,"Завершена")</f>
-        <v/>
-      </c>
-      <c r="I7" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A7,Сделки!$J:$J,"Планируется")</f>
-        <v/>
-      </c>
-      <c r="J7" s="3">
-        <f>COUNTIFS(Сделки!$D:$D,$A7,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$D:$D,$A7,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$D:$D,$A7,Сделки!$J:$J,"Бюджет под риском")</f>
+      <c r="C8" s="5">
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A8)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A8))</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>E8-C8</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>IFERROR(E8/C8,0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>IFERROR(D8/C8,0)</f>
+        <v/>
+      </c>
+      <c r="I8" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="J8" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K8" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L8" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Гоша</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="C9" s="5">
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A9)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A9))</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>E9-C9</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>IFERROR(E9/C9,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>IFERROR(D9/C9,0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="J9" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K9" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L9" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Костя</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="C10" s="5">
+        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A10)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A10))</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>E10-C10</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>IFERROR(E10/C10,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>IFERROR(D10/C10,0)</f>
+        <v/>
+      </c>
+      <c r="I10" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="J10" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <v/>
+      </c>
+      <c r="K10" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <v/>
+      </c>
+      <c r="L10" s="3">
+        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J7"/>
+  <autoFilter ref="A4:L10"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Все,1 квартал,2 квартал,3 квартал,4 квартал"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E100"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Подразделение</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Квартальный план</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Активен</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Петриченко Мария</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Журавлев Иван</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Шатнюк Дарья</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Смирнов Дмитрий</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Гоша</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Годовой план 60 000 000 / 4 квартала</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Костя</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Годовой план 50 000 000 / 4 квартала</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n"/>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n"/>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n"/>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n"/>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="3" t="n"/>
+      <c r="E47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n"/>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="3" t="n"/>
+      <c r="E48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n"/>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="5" t="n"/>
+      <c r="D53" s="3" t="n"/>
+      <c r="E53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n"/>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n"/>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n"/>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="3" t="n"/>
+      <c r="E58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n"/>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n"/>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="3" t="n"/>
+      <c r="E60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n"/>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n"/>
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="3" t="n"/>
+      <c r="E64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n"/>
+      <c r="B65" s="4" t="n"/>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="3" t="n"/>
+      <c r="E65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n"/>
+      <c r="B66" s="4" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n"/>
+      <c r="B67" s="4" t="n"/>
+      <c r="C67" s="5" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n"/>
+      <c r="B68" s="4" t="n"/>
+      <c r="C68" s="5" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n"/>
+      <c r="B69" s="4" t="n"/>
+      <c r="C69" s="5" t="n"/>
+      <c r="D69" s="3" t="n"/>
+      <c r="E69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n"/>
+      <c r="B70" s="4" t="n"/>
+      <c r="C70" s="5" t="n"/>
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n"/>
+      <c r="B71" s="4" t="n"/>
+      <c r="C71" s="5" t="n"/>
+      <c r="D71" s="3" t="n"/>
+      <c r="E71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n"/>
+      <c r="B72" s="4" t="n"/>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="3" t="n"/>
+      <c r="E72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n"/>
+      <c r="B73" s="4" t="n"/>
+      <c r="C73" s="5" t="n"/>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n"/>
+      <c r="B74" s="4" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="3" t="n"/>
+      <c r="E74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n"/>
+      <c r="B75" s="4" t="n"/>
+      <c r="C75" s="5" t="n"/>
+      <c r="D75" s="3" t="n"/>
+      <c r="E75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n"/>
+      <c r="B76" s="4" t="n"/>
+      <c r="C76" s="5" t="n"/>
+      <c r="D76" s="3" t="n"/>
+      <c r="E76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n"/>
+      <c r="B77" s="4" t="n"/>
+      <c r="C77" s="5" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n"/>
+      <c r="B78" s="4" t="n"/>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="3" t="n"/>
+      <c r="E78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n"/>
+      <c r="B79" s="4" t="n"/>
+      <c r="C79" s="5" t="n"/>
+      <c r="D79" s="3" t="n"/>
+      <c r="E79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n"/>
+      <c r="B80" s="4" t="n"/>
+      <c r="C80" s="5" t="n"/>
+      <c r="D80" s="3" t="n"/>
+      <c r="E80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n"/>
+      <c r="B81" s="4" t="n"/>
+      <c r="C81" s="5" t="n"/>
+      <c r="D81" s="3" t="n"/>
+      <c r="E81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n"/>
+      <c r="B82" s="4" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="3" t="n"/>
+      <c r="E82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n"/>
+      <c r="B83" s="4" t="n"/>
+      <c r="C83" s="5" t="n"/>
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n"/>
+      <c r="B84" s="4" t="n"/>
+      <c r="C84" s="5" t="n"/>
+      <c r="D84" s="3" t="n"/>
+      <c r="E84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n"/>
+      <c r="B85" s="4" t="n"/>
+      <c r="C85" s="5" t="n"/>
+      <c r="D85" s="3" t="n"/>
+      <c r="E85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n"/>
+      <c r="B86" s="4" t="n"/>
+      <c r="C86" s="5" t="n"/>
+      <c r="D86" s="3" t="n"/>
+      <c r="E86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n"/>
+      <c r="B87" s="4" t="n"/>
+      <c r="C87" s="5" t="n"/>
+      <c r="D87" s="3" t="n"/>
+      <c r="E87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n"/>
+      <c r="B88" s="4" t="n"/>
+      <c r="C88" s="5" t="n"/>
+      <c r="D88" s="3" t="n"/>
+      <c r="E88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n"/>
+      <c r="B89" s="4" t="n"/>
+      <c r="C89" s="5" t="n"/>
+      <c r="D89" s="3" t="n"/>
+      <c r="E89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n"/>
+      <c r="B90" s="4" t="n"/>
+      <c r="C90" s="5" t="n"/>
+      <c r="D90" s="3" t="n"/>
+      <c r="E90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n"/>
+      <c r="B91" s="4" t="n"/>
+      <c r="C91" s="5" t="n"/>
+      <c r="D91" s="3" t="n"/>
+      <c r="E91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n"/>
+      <c r="B92" s="4" t="n"/>
+      <c r="C92" s="5" t="n"/>
+      <c r="D92" s="3" t="n"/>
+      <c r="E92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n"/>
+      <c r="B93" s="4" t="n"/>
+      <c r="C93" s="5" t="n"/>
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="4" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n"/>
+      <c r="B94" s="4" t="n"/>
+      <c r="C94" s="5" t="n"/>
+      <c r="D94" s="3" t="n"/>
+      <c r="E94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n"/>
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="5" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="4" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n"/>
+      <c r="B96" s="4" t="n"/>
+      <c r="C96" s="5" t="n"/>
+      <c r="D96" s="3" t="n"/>
+      <c r="E96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n"/>
+      <c r="B97" s="4" t="n"/>
+      <c r="C97" s="5" t="n"/>
+      <c r="D97" s="3" t="n"/>
+      <c r="E97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n"/>
+      <c r="B98" s="4" t="n"/>
+      <c r="C98" s="5" t="n"/>
+      <c r="D98" s="3" t="n"/>
+      <c r="E98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n"/>
+      <c r="B99" s="4" t="n"/>
+      <c r="C99" s="5" t="n"/>
+      <c r="D99" s="3" t="n"/>
+      <c r="E99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n"/>
+      <c r="B100" s="4" t="n"/>
+      <c r="C100" s="5" t="n"/>
+      <c r="D100" s="3" t="n"/>
+      <c r="E100" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E100"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Да,Нет"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13805,703 +14033,349 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Виды услуг</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Статусы</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Месяцы</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Кварталы</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>Подразделения</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Сотрудник</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>Подразделение</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Активен</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Комментарий</t>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Квартальный план</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
+        <is>
+          <t>Комментарий к плану</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>SaaS</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Завершена</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Январь</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>1 квартал</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Петриченко Мария</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Данные внесены из предоставленных планов</t>
-        </is>
-      </c>
+      <c r="M2" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="N2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>On-Premise</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Планируется</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Февраль</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>2 квартал</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Журавлев Иван</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Данные внесены из предоставленных планов</t>
-        </is>
-      </c>
+      <c r="M3" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="N3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Услуги</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Обсуждение</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Март</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>3 квартал</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Шатнюк Дарья</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>BI</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Данные внесены из предоставленных планов</t>
-        </is>
-      </c>
+      <c r="M4" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="N4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Доп. план</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Потенциал</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Апрель</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>4 квартал</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Смирнов Дмитрий</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>BI</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Данные внесены из предоставленных планов</t>
-        </is>
-      </c>
+      <c r="M5" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="N5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Up-Sale</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Бюджет под риском</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Май</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Гоша</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Годовой план 60 000 000 / 4 квартала</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Перенесена</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Июнь</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Костя</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Годовой план 50 000 000 / 4 квартала</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Отменена</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Июль</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Август</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Сентябрь</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Октябрь</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Ноябрь</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n"/>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n"/>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="4" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="n"/>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="n"/>
-      <c r="D60" s="4" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-      <c r="D61" s="4" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="n"/>
-      <c r="B62" s="4" t="n"/>
-      <c r="C62" s="4" t="n"/>
-      <c r="D62" s="4" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="4" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="n"/>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-      <c r="D65" s="4" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="n"/>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
-      <c r="D66" s="4" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="n"/>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="n"/>
-      <c r="D67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="n"/>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="n"/>
-      <c r="B69" s="4" t="n"/>
-      <c r="C69" s="4" t="n"/>
-      <c r="D69" s="4" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="n"/>
-      <c r="B70" s="4" t="n"/>
-      <c r="C70" s="4" t="n"/>
-      <c r="D70" s="4" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="n"/>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="n"/>
-      <c r="B72" s="4" t="n"/>
-      <c r="C72" s="4" t="n"/>
-      <c r="D72" s="4" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="n"/>
-      <c r="B73" s="4" t="n"/>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="4" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="n"/>
-      <c r="B74" s="4" t="n"/>
-      <c r="C74" s="4" t="n"/>
-      <c r="D74" s="4" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="n"/>
-      <c r="B75" s="4" t="n"/>
-      <c r="C75" s="4" t="n"/>
-      <c r="D75" s="4" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="n"/>
-      <c r="B76" s="4" t="n"/>
-      <c r="C76" s="4" t="n"/>
-      <c r="D76" s="4" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="n"/>
-      <c r="B77" s="4" t="n"/>
-      <c r="C77" s="4" t="n"/>
-      <c r="D77" s="4" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="n"/>
-      <c r="B78" s="4" t="n"/>
-      <c r="C78" s="4" t="n"/>
-      <c r="D78" s="4" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="n"/>
-      <c r="B79" s="4" t="n"/>
-      <c r="C79" s="4" t="n"/>
-      <c r="D79" s="4" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="n"/>
-      <c r="B80" s="4" t="n"/>
-      <c r="C80" s="4" t="n"/>
-      <c r="D80" s="4" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="n"/>
-      <c r="B81" s="4" t="n"/>
-      <c r="C81" s="4" t="n"/>
-      <c r="D81" s="4" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n"/>
-      <c r="B82" s="4" t="n"/>
-      <c r="C82" s="4" t="n"/>
-      <c r="D82" s="4" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="n"/>
-      <c r="B83" s="4" t="n"/>
-      <c r="C83" s="4" t="n"/>
-      <c r="D83" s="4" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="4" t="n"/>
-      <c r="B84" s="4" t="n"/>
-      <c r="C84" s="4" t="n"/>
-      <c r="D84" s="4" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="n"/>
-      <c r="B85" s="4" t="n"/>
-      <c r="C85" s="4" t="n"/>
-      <c r="D85" s="4" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="n"/>
-      <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="n"/>
-      <c r="D86" s="4" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="n"/>
-      <c r="B87" s="4" t="n"/>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="4" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="4" t="n"/>
-      <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="n"/>
-      <c r="D88" s="4" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="4" t="n"/>
-      <c r="B89" s="4" t="n"/>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="4" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="n"/>
-      <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="4" t="n"/>
-      <c r="B91" s="4" t="n"/>
-      <c r="C91" s="4" t="n"/>
-      <c r="D91" s="4" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="n"/>
-      <c r="B92" s="4" t="n"/>
-      <c r="C92" s="4" t="n"/>
-      <c r="D92" s="4" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="n"/>
-      <c r="B93" s="4" t="n"/>
-      <c r="C93" s="4" t="n"/>
-      <c r="D93" s="4" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="n"/>
-      <c r="B94" s="4" t="n"/>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="4" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="n"/>
-      <c r="B95" s="4" t="n"/>
-      <c r="C95" s="4" t="n"/>
-      <c r="D95" s="4" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="4" t="n"/>
-      <c r="B96" s="4" t="n"/>
-      <c r="C96" s="4" t="n"/>
-      <c r="D96" s="4" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="4" t="n"/>
-      <c r="B97" s="4" t="n"/>
-      <c r="C97" s="4" t="n"/>
-      <c r="D97" s="4" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="n"/>
-      <c r="B98" s="4" t="n"/>
-      <c r="C98" s="4" t="n"/>
-      <c r="D98" s="4" t="n"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="n"/>
-      <c r="B99" s="4" t="n"/>
-      <c r="C99" s="4" t="n"/>
-      <c r="D99" s="4" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="4" t="n"/>
-      <c r="B100" s="4" t="n"/>
-      <c r="C100" s="4" t="n"/>
-      <c r="D100" s="4" t="n"/>
-    </row>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Декабрь</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
-  <autoFilter ref="A1:D100"/>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Да,Нет"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <autoFilter ref="A1:N20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -14511,245 +14385,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Виды услуг</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>Статусы</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>Месяцы</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>Кварталы</t>
-        </is>
-      </c>
-      <c r="I1" s="11" t="inlineStr">
-        <is>
-          <t>Подразделения</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>SaaS</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Завершена</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Январь</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>1 квартал</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>On-Premise</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Планируется</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Февраль</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>2 квартал</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>BI</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Услуги</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Обсуждение</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Март</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>3 квартал</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Доп. план</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Потенциал</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Апрель</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>4 квартал</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Up-Sale</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Бюджет под риском</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Май</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Перенесена</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Июнь</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Отменена</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Июль</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Август</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Сентябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Октябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Ноябрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Декабрь</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-  </sheetData>
-  <autoFilter ref="A1:I20"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14760,7 +14404,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Фильтры</t>
         </is>
@@ -14801,16 +14445,16 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>План компании</t>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>План</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$H$2:$H$500)</f>
-        <v/>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+        <f>IF($C$3="Все",SUM(Справочники!$M$2:$M$7)*4,SUM(Справочники!$M$2:$M$7))</f>
+        <v/>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Сделок всего</t>
         </is>
@@ -14821,16 +14465,16 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Факт</t>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Прогноз</t>
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Завершено</t>
         </is>
@@ -14841,16 +14485,16 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Отклонение</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Факт</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>B7-B6</f>
-        <v/>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Планируется</t>
         </is>
@@ -14861,22 +14505,33 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Выполнение</t>
-        </is>
-      </c>
-      <c r="B9" s="10">
-        <f>IFERROR(B7/B6,0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Выполнение факта</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>IFERROR(B8/B6,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Обсуждение/риски</t>
         </is>
       </c>
       <c r="E9" s="5">
         <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Покрытие планов прогнозом</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>IFERROR(B7/B6,0)</f>
         <v/>
       </c>
     </row>
@@ -14893,5 +14548,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correct quarterly employee plan summary
Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sales_plan_company_filled.xlsx
+++ b/sales_plan_company_filled.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сделки'!$A$1:$N$500</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сводка по сотрудникам'!$A$4:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сводка по сотрудникам'!$A$3:$R$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Источники'!$A$1:$E$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Справочники'!$A$1:$N$20</definedName>
   </definedNames>
@@ -128,9 +128,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -141,6 +138,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -262,12 +262,7 @@
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Суммы из индивидуальных планов сотрудников. По уточнению это прогноз/пайплайн, не целевой план.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Вероятность оставлена как справочный признак для ясности, без дополнительных расчетов.</t>
+        <t>Суммы из индивидуальных планов сотрудников. Это прогноз/пайплайн, а не целевой план.</t>
       </text>
     </comment>
   </commentList>
@@ -280,14 +275,9 @@
     <author>Cursor</author>
   </authors>
   <commentList>
-    <comment ref="C4" authorId="0" shapeId="0">
+    <comment ref="C3" authorId="0" shapeId="0">
       <text>
-        <t>Если выбран конкретный квартал — план за квартал. Если выбрано Все — годовой план как 4 квартала.</t>
-      </text>
-    </comment>
-    <comment ref="D4" authorId="0" shapeId="0">
-      <text>
-        <t>Сумма из листа Сделки; по уточнению это прогноз/пайплайн.</t>
+        <t>Квартальный план показывается как квартальная цифра. В этой сводке нет умножения на 4.</t>
       </text>
     </comment>
   </commentList>
@@ -302,7 +292,7 @@
   <commentList>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Настоящий план сотрудника на квартал. Суммы из листа Сделки считаются прогнозом/пайплайном.</t>
+        <t>Квартальный план сотрудника. Эти цифры не умножаются в сводке по сотрудникам.</t>
       </text>
     </comment>
   </commentList>
@@ -315,9 +305,9 @@
     <author>Cursor</author>
   </authors>
   <commentList>
-    <comment ref="B7" authorId="0" shapeId="0">
+    <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Прогноз — это суммы из листа Сделки.</t>
+        <t>Сумма квартальных планов сотрудников. Без пересчета в год.</t>
       </text>
     </comment>
   </commentList>
@@ -12763,108 +12753,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Сводка по сотрудникам</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Фильтр по кварталу</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Все</t>
+          <t>Сводка по сотрудникам: выполнение планов поквартально</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Сотрудник</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Подразделение</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>1 квартал план</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>1 квартал прогноз</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>1 квартал факт</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>1 квартал выполнение</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>2 квартал план</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>2 квартал прогноз</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>2 квартал факт</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>2 квартал выполнение</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>3 квартал план</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>3 квартал прогноз</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>3 квартал факт</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>3 квартал выполнение</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>4 квартал план</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>4 квартал прогноз</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>4 квартал факт</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>4 квартал выполнение</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Сотрудник</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Подразделение</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Квартальный план</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Прогноз</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Факт</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Отклонение факт-план</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>Выполнение факта, %</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>Выполнение прогноза, %</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>Сделок всего</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>Завершено</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>В работе</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr">
-        <is>
-          <t>Обсуждение/риски</t>
-        </is>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Петриченко Мария</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="D4" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A4,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A4,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F4" s="8">
+        <f>IFERROR(E4/C4,0)</f>
+        <v/>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="H4" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A4,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A4,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J4" s="8">
+        <f>IFERROR(I4/G4,0)</f>
+        <v/>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="L4" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A4,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M4" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A4,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N4" s="8">
+        <f>IFERROR(M4/K4,0)</f>
+        <v/>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="P4" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A4,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q4" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A4,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R4" s="8">
+        <f>IFERROR(Q4/O4,0)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Петриченко Мария</t>
+          <t>Журавлев Иван</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -12872,103 +12958,143 @@
           <t>SP</t>
         </is>
       </c>
-      <c r="C5" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A5)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A5))</f>
-        <v/>
+      <c r="C5" s="5" t="n">
+        <v>1500000</v>
       </c>
       <c r="D5" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*Сделки!$H$2:$H$500)</f>
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A5,Сделки!$B:$B,"1 квартал")</f>
         <v/>
       </c>
       <c r="E5" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F5" s="5">
-        <f>E5-C5</f>
-        <v/>
-      </c>
-      <c r="G5" s="9">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A5,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F5" s="8">
         <f>IFERROR(E5/C5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="9">
-        <f>IFERROR(D5/C5,0)</f>
-        <v/>
-      </c>
-      <c r="I5" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J5" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K5" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L5" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A5)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+      <c r="G5" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="H5" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A5,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A5,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J5" s="8">
+        <f>IFERROR(I5/G5,0)</f>
+        <v/>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="L5" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A5,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M5" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A5,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N5" s="8">
+        <f>IFERROR(M5/K5,0)</f>
+        <v/>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="P5" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A5,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q5" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A5,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R5" s="8">
+        <f>IFERROR(Q5/O5,0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Журавлев Иван</t>
+          <t>Шатнюк Дарья</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="C6" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A6)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A6))</f>
-        <v/>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>5000000</v>
       </c>
       <c r="D6" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*Сделки!$H$2:$H$500)</f>
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A6,Сделки!$B:$B,"1 квартал")</f>
         <v/>
       </c>
       <c r="E6" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>E6-C6</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A6,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F6" s="8">
         <f>IFERROR(E6/C6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="9">
-        <f>IFERROR(D6/C6,0)</f>
-        <v/>
-      </c>
-      <c r="I6" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J6" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K6" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L6" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A6)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+      <c r="G6" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H6" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A6,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A6,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J6" s="8">
+        <f>IFERROR(I6/G6,0)</f>
+        <v/>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L6" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A6,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M6" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A6,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N6" s="8">
+        <f>IFERROR(M6/K6,0)</f>
+        <v/>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="P6" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A6,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q6" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A6,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R6" s="8">
+        <f>IFERROR(Q6/O6,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Шатнюк Дарья</t>
+          <t>Смирнов Дмитрий</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -12976,103 +13102,143 @@
           <t>BI</t>
         </is>
       </c>
-      <c r="C7" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A7)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A7))</f>
-        <v/>
+      <c r="C7" s="5" t="n">
+        <v>5000000</v>
       </c>
       <c r="D7" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*Сделки!$H$2:$H$500)</f>
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A7,Сделки!$B:$B,"1 квартал")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>E7-C7</f>
-        <v/>
-      </c>
-      <c r="G7" s="9">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A7,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F7" s="8">
         <f>IFERROR(E7/C7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="9">
-        <f>IFERROR(D7/C7,0)</f>
-        <v/>
-      </c>
-      <c r="I7" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J7" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K7" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L7" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A7)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+      <c r="G7" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="H7" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A7,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A7,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J7" s="8">
+        <f>IFERROR(I7/G7,0)</f>
+        <v/>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L7" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A7,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M7" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A7,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N7" s="8">
+        <f>IFERROR(M7/K7,0)</f>
+        <v/>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="P7" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A7,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A7,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R7" s="8">
+        <f>IFERROR(Q7/O7,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Смирнов Дмитрий</t>
+          <t>Гоша</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>BI</t>
-        </is>
-      </c>
-      <c r="C8" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A8)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A8))</f>
-        <v/>
+          <t>Не указано</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>15000000</v>
       </c>
       <c r="D8" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*Сделки!$H$2:$H$500)</f>
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"1 квартал")</f>
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>E8-C8</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A8,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
         <f>IFERROR(E8/C8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="9">
-        <f>IFERROR(D8/C8,0)</f>
-        <v/>
-      </c>
-      <c r="I8" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J8" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K8" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L8" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A8)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+      <c r="G8" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="H8" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A8,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J8" s="8">
+        <f>IFERROR(I8/G8,0)</f>
+        <v/>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L8" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M8" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A8,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N8" s="8">
+        <f>IFERROR(M8/K8,0)</f>
+        <v/>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="P8" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q8" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A8,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R8" s="8">
+        <f>IFERROR(Q8/O8,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Гоша</t>
+          <t>Костя</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -13080,109 +13246,72 @@
           <t>Не указано</t>
         </is>
       </c>
-      <c r="C9" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A9)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A9))</f>
-        <v/>
+      <c r="C9" s="5" t="n">
+        <v>12500000</v>
       </c>
       <c r="D9" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*Сделки!$H$2:$H$500)</f>
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"1 квартал")</f>
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>E9-C9</f>
-        <v/>
-      </c>
-      <c r="G9" s="9">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A9,Сделки!$B:$B,"1 квартал")</f>
+        <v/>
+      </c>
+      <c r="F9" s="8">
         <f>IFERROR(E9/C9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="9">
-        <f>IFERROR(D9/C9,0)</f>
-        <v/>
-      </c>
-      <c r="I9" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J9" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K9" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L9" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A9)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Костя</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Не указано</t>
-        </is>
-      </c>
-      <c r="C10" s="5">
-        <f>IF($B$2="Все",SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A10)*4,SUMIFS(Справочники!$M:$M,Справочники!$K:$K,$A10))</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*Сделки!$H$2:$H$500)</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="F10" s="5">
-        <f>E10-C10</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
-        <f>IFERROR(E10/C10,0)</f>
-        <v/>
-      </c>
-      <c r="H10" s="9">
-        <f>IFERROR(D10/C10,0)</f>
-        <v/>
-      </c>
-      <c r="I10" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="J10" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$J$2:$J$500="Завершена"))</f>
-        <v/>
-      </c>
-      <c r="K10" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*(Сделки!$J$2:$J$500="Планируется"))</f>
-        <v/>
-      </c>
-      <c r="L10" s="3">
-        <f>SUMPRODUCT(IF($B$2="Все",1,--(Сделки!$B$2:$B$500=$B$2))*(Сделки!$D$2:$D$500=$A10)*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+      <c r="G9" s="5" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="H9" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="I9" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A9,Сделки!$B:$B,"2 квартал")</f>
+        <v/>
+      </c>
+      <c r="J9" s="8">
+        <f>IFERROR(I9/G9,0)</f>
+        <v/>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="L9" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="M9" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A9,Сделки!$B:$B,"3 квартал")</f>
+        <v/>
+      </c>
+      <c r="N9" s="8">
+        <f>IFERROR(M9/K9,0)</f>
+        <v/>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>12500000</v>
+      </c>
+      <c r="P9" s="5">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="Q9" s="5">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$D:$D,$A9,Сделки!$B:$B,"4 квартал")</f>
+        <v/>
+      </c>
+      <c r="R9" s="8">
+        <f>IFERROR(Q9/O9,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L10"/>
+  <autoFilter ref="A3:R9"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Все,1 квартал,2 квартал,3 квартал,4 квартал"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -13201,7 +13330,7 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13243,7 +13372,7 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>1000000</v>
+        <v>1500000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
@@ -13336,7 +13465,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 60 000 000 / 4 квартала</t>
+          <t>Годовой план 60 000 000, квартальный 15 000 000</t>
         </is>
       </c>
     </row>
@@ -13361,7 +13490,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 50 000 000 / 4 квартала</t>
+          <t>Годовой план 50 000 000, квартальный 12 500 000</t>
         </is>
       </c>
     </row>
@@ -14044,53 +14173,53 @@
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Виды услуг</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Статусы</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Месяцы</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Кварталы</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Подразделения</t>
         </is>
       </c>
-      <c r="K1" s="11" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Сотрудник</t>
         </is>
       </c>
-      <c r="L1" s="11" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>Подразделение</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>Квартальный план</t>
         </is>
       </c>
-      <c r="N1" s="11" t="inlineStr">
-        <is>
-          <t>Комментарий к плану</t>
+      <c r="N1" s="10" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
         </is>
       </c>
     </row>
@@ -14131,7 +14260,7 @@
         </is>
       </c>
       <c r="M2" s="5" t="n">
-        <v>1000000</v>
+        <v>1500000</v>
       </c>
       <c r="N2" s="4" t="inlineStr"/>
     </row>
@@ -14284,7 +14413,7 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 60 000 000 / 4 квартала</t>
+          <t>Годовой план 60 000 000, квартальный 15 000 000</t>
         </is>
       </c>
     </row>
@@ -14314,7 +14443,7 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 50 000 000 / 4 квартала</t>
+          <t>Годовой план 50 000 000, квартальный 12 500 000</t>
         </is>
       </c>
     </row>
@@ -14397,14 +14526,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Дашборд продаж</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Фильтры</t>
         </is>
@@ -14427,7 +14556,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Все</t>
+          <t>2 квартал</t>
         </is>
       </c>
     </row>
@@ -14445,92 +14574,92 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>План</t>
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>План на квартал</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>IF($C$3="Все",SUM(Справочники!$M$2:$M$7)*4,SUM(Справочники!$M$2:$M$7))</f>
-        <v/>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+        <f>SUM(Справочники!$M$2:$M$7)</f>
+        <v/>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Сделок всего</t>
         </is>
       </c>
       <c r="E6" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$F$2:$F$500&lt;&gt;""))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Прогноз</t>
         </is>
       </c>
       <c r="B7" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$H$2:$H$500)</f>
-        <v/>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$H$2:$H$500)</f>
+        <v/>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Завершено</t>
         </is>
       </c>
       <c r="E7" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$J$2:$J$500="Завершена"))</f>
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$J$2:$J$500="Завершена"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Факт</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$I$2:$I$500)</f>
-        <v/>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*Сделки!$I$2:$I$500)</f>
+        <v/>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Планируется</t>
         </is>
       </c>
       <c r="E8" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$J$2:$J$500="Планируется"))</f>
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*(Сделки!$J$2:$J$500="Планируется"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Выполнение факта</t>
         </is>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <f>IFERROR(B8/B6,0)</f>
         <v/>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Обсуждение/риски</t>
         </is>
       </c>
       <c r="E9" s="5">
-        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*IF($C$3="Все",1,--(Сделки!$B$2:$B$500=$C$3))*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
+        <f>SUMPRODUCT((Сделки!$A$2:$A$500=$C$2)*(Сделки!$B$2:$B$500=$C$3)*IF($C$4="Все",1,--(Сделки!$C$2:$C$500=$C$4))*((Сделки!$J$2:$J$500="Обсуждение")+(Сделки!$J$2:$J$500="Потенциал")+(Сделки!$J$2:$J$500="Бюджет под риском")))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Покрытие планов прогнозом</t>
         </is>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="8">
         <f>IFERROR(B7/B6,0)</f>
         <v/>
       </c>
@@ -14541,7 +14670,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Все,1 квартал,2 квартал,3 квартал,4 квартал"</formula1>
+      <formula1>"1 квартал,2 квартал,3 квартал,4 квартал"</formula1>
     </dataValidation>
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Все,Январь,Февраль,Март,Апрель,Май,Июнь,Июль,Август,Сентябрь,Октябрь,Ноябрь,Декабрь"</formula1>

</xml_diff>

<commit_message>
Fix quarterly targets for dashboard
Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sales_plan_company_filled.xlsx
+++ b/sales_plan_company_filled.xlsx
@@ -25,9 +25,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -107,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,7 +123,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +138,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -293,21 +295,6 @@
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Квартальный план сотрудника. Эти цифры не умножаются в сводке по сотрудникам.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Cursor</author>
-  </authors>
-  <commentList>
-    <comment ref="B6" authorId="0" shapeId="0">
-      <text>
-        <t>Сумма квартальных планов сотрудников. Без пересчета в год.</t>
       </text>
     </comment>
   </commentList>
@@ -772,7 +759,7 @@
         <v/>
       </c>
       <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="6" t="n">
+      <c r="N2" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -831,7 +818,7 @@
         <v/>
       </c>
       <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="6" t="n">
+      <c r="N3" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -890,7 +877,7 @@
         <v/>
       </c>
       <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -949,7 +936,7 @@
         <v/>
       </c>
       <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="6" t="n">
+      <c r="N5" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1008,7 +995,7 @@
         <v/>
       </c>
       <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="6" t="n">
+      <c r="N6" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1067,7 +1054,7 @@
         <v/>
       </c>
       <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="6" t="n">
+      <c r="N7" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1126,7 +1113,7 @@
         <v/>
       </c>
       <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="6" t="n">
+      <c r="N8" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1185,7 +1172,7 @@
         <v/>
       </c>
       <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="6" t="n">
+      <c r="N9" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1244,7 +1231,7 @@
         <v/>
       </c>
       <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="6" t="n">
+      <c r="N10" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1303,7 +1290,7 @@
         <v/>
       </c>
       <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="6" t="n">
+      <c r="N11" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1362,7 +1349,7 @@
         <v/>
       </c>
       <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="6" t="n">
+      <c r="N12" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1421,7 +1408,7 @@
         <v/>
       </c>
       <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="6" t="n">
+      <c r="N13" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1480,7 +1467,7 @@
         <v/>
       </c>
       <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="6" t="n">
+      <c r="N14" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1539,7 +1526,7 @@
         <v/>
       </c>
       <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="6" t="n">
+      <c r="N15" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1598,7 +1585,7 @@
         <v/>
       </c>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="6" t="n">
+      <c r="N16" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1657,7 +1644,7 @@
         <v/>
       </c>
       <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="6" t="n">
+      <c r="N17" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1716,7 +1703,7 @@
         <v/>
       </c>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="6" t="n">
+      <c r="N18" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1775,7 +1762,7 @@
         <v/>
       </c>
       <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="6" t="n">
+      <c r="N19" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1834,7 +1821,7 @@
         <v/>
       </c>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="6" t="n">
+      <c r="N20" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1893,7 +1880,7 @@
         <v/>
       </c>
       <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" s="6" t="n">
+      <c r="N21" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -1952,7 +1939,7 @@
         <v/>
       </c>
       <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="6" t="n">
+      <c r="N22" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2011,7 +1998,7 @@
         <v/>
       </c>
       <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="6" t="n">
+      <c r="N23" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2070,7 +2057,7 @@
         <v/>
       </c>
       <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="6" t="n">
+      <c r="N24" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2129,7 +2116,7 @@
         <v/>
       </c>
       <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="6" t="n">
+      <c r="N25" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2188,7 +2175,7 @@
         <v/>
       </c>
       <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="6" t="n">
+      <c r="N26" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2247,7 +2234,7 @@
         <v/>
       </c>
       <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="6" t="n">
+      <c r="N27" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2306,7 +2293,7 @@
         <v/>
       </c>
       <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="6" t="n">
+      <c r="N28" s="13" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -2327,7 +2314,7 @@
         <v/>
       </c>
       <c r="M29" s="4" t="n"/>
-      <c r="N29" s="6">
+      <c r="N29" s="13">
         <f>IF(A29="","",TODAY())</f>
         <v/>
       </c>
@@ -2349,7 +2336,7 @@
         <v/>
       </c>
       <c r="M30" s="4" t="n"/>
-      <c r="N30" s="6">
+      <c r="N30" s="13">
         <f>IF(A30="","",TODAY())</f>
         <v/>
       </c>
@@ -2371,7 +2358,7 @@
         <v/>
       </c>
       <c r="M31" s="4" t="n"/>
-      <c r="N31" s="6">
+      <c r="N31" s="13">
         <f>IF(A31="","",TODAY())</f>
         <v/>
       </c>
@@ -2393,7 +2380,7 @@
         <v/>
       </c>
       <c r="M32" s="4" t="n"/>
-      <c r="N32" s="6">
+      <c r="N32" s="13">
         <f>IF(A32="","",TODAY())</f>
         <v/>
       </c>
@@ -2415,7 +2402,7 @@
         <v/>
       </c>
       <c r="M33" s="4" t="n"/>
-      <c r="N33" s="6">
+      <c r="N33" s="13">
         <f>IF(A33="","",TODAY())</f>
         <v/>
       </c>
@@ -2437,7 +2424,7 @@
         <v/>
       </c>
       <c r="M34" s="4" t="n"/>
-      <c r="N34" s="6">
+      <c r="N34" s="13">
         <f>IF(A34="","",TODAY())</f>
         <v/>
       </c>
@@ -2459,7 +2446,7 @@
         <v/>
       </c>
       <c r="M35" s="4" t="n"/>
-      <c r="N35" s="6">
+      <c r="N35" s="13">
         <f>IF(A35="","",TODAY())</f>
         <v/>
       </c>
@@ -2481,7 +2468,7 @@
         <v/>
       </c>
       <c r="M36" s="4" t="n"/>
-      <c r="N36" s="6">
+      <c r="N36" s="13">
         <f>IF(A36="","",TODAY())</f>
         <v/>
       </c>
@@ -2503,7 +2490,7 @@
         <v/>
       </c>
       <c r="M37" s="4" t="n"/>
-      <c r="N37" s="6">
+      <c r="N37" s="13">
         <f>IF(A37="","",TODAY())</f>
         <v/>
       </c>
@@ -2525,7 +2512,7 @@
         <v/>
       </c>
       <c r="M38" s="4" t="n"/>
-      <c r="N38" s="6">
+      <c r="N38" s="13">
         <f>IF(A38="","",TODAY())</f>
         <v/>
       </c>
@@ -2547,7 +2534,7 @@
         <v/>
       </c>
       <c r="M39" s="4" t="n"/>
-      <c r="N39" s="6">
+      <c r="N39" s="13">
         <f>IF(A39="","",TODAY())</f>
         <v/>
       </c>
@@ -2569,7 +2556,7 @@
         <v/>
       </c>
       <c r="M40" s="4" t="n"/>
-      <c r="N40" s="6">
+      <c r="N40" s="13">
         <f>IF(A40="","",TODAY())</f>
         <v/>
       </c>
@@ -2591,7 +2578,7 @@
         <v/>
       </c>
       <c r="M41" s="4" t="n"/>
-      <c r="N41" s="6">
+      <c r="N41" s="13">
         <f>IF(A41="","",TODAY())</f>
         <v/>
       </c>
@@ -2613,7 +2600,7 @@
         <v/>
       </c>
       <c r="M42" s="4" t="n"/>
-      <c r="N42" s="6">
+      <c r="N42" s="13">
         <f>IF(A42="","",TODAY())</f>
         <v/>
       </c>
@@ -2635,7 +2622,7 @@
         <v/>
       </c>
       <c r="M43" s="4" t="n"/>
-      <c r="N43" s="6">
+      <c r="N43" s="13">
         <f>IF(A43="","",TODAY())</f>
         <v/>
       </c>
@@ -2657,7 +2644,7 @@
         <v/>
       </c>
       <c r="M44" s="4" t="n"/>
-      <c r="N44" s="6">
+      <c r="N44" s="13">
         <f>IF(A44="","",TODAY())</f>
         <v/>
       </c>
@@ -2679,7 +2666,7 @@
         <v/>
       </c>
       <c r="M45" s="4" t="n"/>
-      <c r="N45" s="6">
+      <c r="N45" s="13">
         <f>IF(A45="","",TODAY())</f>
         <v/>
       </c>
@@ -2701,7 +2688,7 @@
         <v/>
       </c>
       <c r="M46" s="4" t="n"/>
-      <c r="N46" s="6">
+      <c r="N46" s="13">
         <f>IF(A46="","",TODAY())</f>
         <v/>
       </c>
@@ -2723,7 +2710,7 @@
         <v/>
       </c>
       <c r="M47" s="4" t="n"/>
-      <c r="N47" s="6">
+      <c r="N47" s="13">
         <f>IF(A47="","",TODAY())</f>
         <v/>
       </c>
@@ -2745,7 +2732,7 @@
         <v/>
       </c>
       <c r="M48" s="4" t="n"/>
-      <c r="N48" s="6">
+      <c r="N48" s="13">
         <f>IF(A48="","",TODAY())</f>
         <v/>
       </c>
@@ -2767,7 +2754,7 @@
         <v/>
       </c>
       <c r="M49" s="4" t="n"/>
-      <c r="N49" s="6">
+      <c r="N49" s="13">
         <f>IF(A49="","",TODAY())</f>
         <v/>
       </c>
@@ -2789,7 +2776,7 @@
         <v/>
       </c>
       <c r="M50" s="4" t="n"/>
-      <c r="N50" s="6">
+      <c r="N50" s="13">
         <f>IF(A50="","",TODAY())</f>
         <v/>
       </c>
@@ -2811,7 +2798,7 @@
         <v/>
       </c>
       <c r="M51" s="4" t="n"/>
-      <c r="N51" s="6">
+      <c r="N51" s="13">
         <f>IF(A51="","",TODAY())</f>
         <v/>
       </c>
@@ -2833,7 +2820,7 @@
         <v/>
       </c>
       <c r="M52" s="4" t="n"/>
-      <c r="N52" s="6">
+      <c r="N52" s="13">
         <f>IF(A52="","",TODAY())</f>
         <v/>
       </c>
@@ -2855,7 +2842,7 @@
         <v/>
       </c>
       <c r="M53" s="4" t="n"/>
-      <c r="N53" s="6">
+      <c r="N53" s="13">
         <f>IF(A53="","",TODAY())</f>
         <v/>
       </c>
@@ -2877,7 +2864,7 @@
         <v/>
       </c>
       <c r="M54" s="4" t="n"/>
-      <c r="N54" s="6">
+      <c r="N54" s="13">
         <f>IF(A54="","",TODAY())</f>
         <v/>
       </c>
@@ -2899,7 +2886,7 @@
         <v/>
       </c>
       <c r="M55" s="4" t="n"/>
-      <c r="N55" s="6">
+      <c r="N55" s="13">
         <f>IF(A55="","",TODAY())</f>
         <v/>
       </c>
@@ -2921,7 +2908,7 @@
         <v/>
       </c>
       <c r="M56" s="4" t="n"/>
-      <c r="N56" s="6">
+      <c r="N56" s="13">
         <f>IF(A56="","",TODAY())</f>
         <v/>
       </c>
@@ -2943,7 +2930,7 @@
         <v/>
       </c>
       <c r="M57" s="4" t="n"/>
-      <c r="N57" s="6">
+      <c r="N57" s="13">
         <f>IF(A57="","",TODAY())</f>
         <v/>
       </c>
@@ -2965,7 +2952,7 @@
         <v/>
       </c>
       <c r="M58" s="4" t="n"/>
-      <c r="N58" s="6">
+      <c r="N58" s="13">
         <f>IF(A58="","",TODAY())</f>
         <v/>
       </c>
@@ -2987,7 +2974,7 @@
         <v/>
       </c>
       <c r="M59" s="4" t="n"/>
-      <c r="N59" s="6">
+      <c r="N59" s="13">
         <f>IF(A59="","",TODAY())</f>
         <v/>
       </c>
@@ -3009,7 +2996,7 @@
         <v/>
       </c>
       <c r="M60" s="4" t="n"/>
-      <c r="N60" s="6">
+      <c r="N60" s="13">
         <f>IF(A60="","",TODAY())</f>
         <v/>
       </c>
@@ -3031,7 +3018,7 @@
         <v/>
       </c>
       <c r="M61" s="4" t="n"/>
-      <c r="N61" s="6">
+      <c r="N61" s="13">
         <f>IF(A61="","",TODAY())</f>
         <v/>
       </c>
@@ -3053,7 +3040,7 @@
         <v/>
       </c>
       <c r="M62" s="4" t="n"/>
-      <c r="N62" s="6">
+      <c r="N62" s="13">
         <f>IF(A62="","",TODAY())</f>
         <v/>
       </c>
@@ -3075,7 +3062,7 @@
         <v/>
       </c>
       <c r="M63" s="4" t="n"/>
-      <c r="N63" s="6">
+      <c r="N63" s="13">
         <f>IF(A63="","",TODAY())</f>
         <v/>
       </c>
@@ -3097,7 +3084,7 @@
         <v/>
       </c>
       <c r="M64" s="4" t="n"/>
-      <c r="N64" s="6">
+      <c r="N64" s="13">
         <f>IF(A64="","",TODAY())</f>
         <v/>
       </c>
@@ -3119,7 +3106,7 @@
         <v/>
       </c>
       <c r="M65" s="4" t="n"/>
-      <c r="N65" s="6">
+      <c r="N65" s="13">
         <f>IF(A65="","",TODAY())</f>
         <v/>
       </c>
@@ -3141,7 +3128,7 @@
         <v/>
       </c>
       <c r="M66" s="4" t="n"/>
-      <c r="N66" s="6">
+      <c r="N66" s="13">
         <f>IF(A66="","",TODAY())</f>
         <v/>
       </c>
@@ -3163,7 +3150,7 @@
         <v/>
       </c>
       <c r="M67" s="4" t="n"/>
-      <c r="N67" s="6">
+      <c r="N67" s="13">
         <f>IF(A67="","",TODAY())</f>
         <v/>
       </c>
@@ -3185,7 +3172,7 @@
         <v/>
       </c>
       <c r="M68" s="4" t="n"/>
-      <c r="N68" s="6">
+      <c r="N68" s="13">
         <f>IF(A68="","",TODAY())</f>
         <v/>
       </c>
@@ -3207,7 +3194,7 @@
         <v/>
       </c>
       <c r="M69" s="4" t="n"/>
-      <c r="N69" s="6">
+      <c r="N69" s="13">
         <f>IF(A69="","",TODAY())</f>
         <v/>
       </c>
@@ -3229,7 +3216,7 @@
         <v/>
       </c>
       <c r="M70" s="4" t="n"/>
-      <c r="N70" s="6">
+      <c r="N70" s="13">
         <f>IF(A70="","",TODAY())</f>
         <v/>
       </c>
@@ -3251,7 +3238,7 @@
         <v/>
       </c>
       <c r="M71" s="4" t="n"/>
-      <c r="N71" s="6">
+      <c r="N71" s="13">
         <f>IF(A71="","",TODAY())</f>
         <v/>
       </c>
@@ -3273,7 +3260,7 @@
         <v/>
       </c>
       <c r="M72" s="4" t="n"/>
-      <c r="N72" s="6">
+      <c r="N72" s="13">
         <f>IF(A72="","",TODAY())</f>
         <v/>
       </c>
@@ -3295,7 +3282,7 @@
         <v/>
       </c>
       <c r="M73" s="4" t="n"/>
-      <c r="N73" s="6">
+      <c r="N73" s="13">
         <f>IF(A73="","",TODAY())</f>
         <v/>
       </c>
@@ -3317,7 +3304,7 @@
         <v/>
       </c>
       <c r="M74" s="4" t="n"/>
-      <c r="N74" s="6">
+      <c r="N74" s="13">
         <f>IF(A74="","",TODAY())</f>
         <v/>
       </c>
@@ -3339,7 +3326,7 @@
         <v/>
       </c>
       <c r="M75" s="4" t="n"/>
-      <c r="N75" s="6">
+      <c r="N75" s="13">
         <f>IF(A75="","",TODAY())</f>
         <v/>
       </c>
@@ -3361,7 +3348,7 @@
         <v/>
       </c>
       <c r="M76" s="4" t="n"/>
-      <c r="N76" s="6">
+      <c r="N76" s="13">
         <f>IF(A76="","",TODAY())</f>
         <v/>
       </c>
@@ -3383,7 +3370,7 @@
         <v/>
       </c>
       <c r="M77" s="4" t="n"/>
-      <c r="N77" s="6">
+      <c r="N77" s="13">
         <f>IF(A77="","",TODAY())</f>
         <v/>
       </c>
@@ -3405,7 +3392,7 @@
         <v/>
       </c>
       <c r="M78" s="4" t="n"/>
-      <c r="N78" s="6">
+      <c r="N78" s="13">
         <f>IF(A78="","",TODAY())</f>
         <v/>
       </c>
@@ -3427,7 +3414,7 @@
         <v/>
       </c>
       <c r="M79" s="4" t="n"/>
-      <c r="N79" s="6">
+      <c r="N79" s="13">
         <f>IF(A79="","",TODAY())</f>
         <v/>
       </c>
@@ -3449,7 +3436,7 @@
         <v/>
       </c>
       <c r="M80" s="4" t="n"/>
-      <c r="N80" s="6">
+      <c r="N80" s="13">
         <f>IF(A80="","",TODAY())</f>
         <v/>
       </c>
@@ -3471,7 +3458,7 @@
         <v/>
       </c>
       <c r="M81" s="4" t="n"/>
-      <c r="N81" s="6">
+      <c r="N81" s="13">
         <f>IF(A81="","",TODAY())</f>
         <v/>
       </c>
@@ -3493,7 +3480,7 @@
         <v/>
       </c>
       <c r="M82" s="4" t="n"/>
-      <c r="N82" s="6">
+      <c r="N82" s="13">
         <f>IF(A82="","",TODAY())</f>
         <v/>
       </c>
@@ -3515,7 +3502,7 @@
         <v/>
       </c>
       <c r="M83" s="4" t="n"/>
-      <c r="N83" s="6">
+      <c r="N83" s="13">
         <f>IF(A83="","",TODAY())</f>
         <v/>
       </c>
@@ -3537,7 +3524,7 @@
         <v/>
       </c>
       <c r="M84" s="4" t="n"/>
-      <c r="N84" s="6">
+      <c r="N84" s="13">
         <f>IF(A84="","",TODAY())</f>
         <v/>
       </c>
@@ -3559,7 +3546,7 @@
         <v/>
       </c>
       <c r="M85" s="4" t="n"/>
-      <c r="N85" s="6">
+      <c r="N85" s="13">
         <f>IF(A85="","",TODAY())</f>
         <v/>
       </c>
@@ -3581,7 +3568,7 @@
         <v/>
       </c>
       <c r="M86" s="4" t="n"/>
-      <c r="N86" s="6">
+      <c r="N86" s="13">
         <f>IF(A86="","",TODAY())</f>
         <v/>
       </c>
@@ -3603,7 +3590,7 @@
         <v/>
       </c>
       <c r="M87" s="4" t="n"/>
-      <c r="N87" s="6">
+      <c r="N87" s="13">
         <f>IF(A87="","",TODAY())</f>
         <v/>
       </c>
@@ -3625,7 +3612,7 @@
         <v/>
       </c>
       <c r="M88" s="4" t="n"/>
-      <c r="N88" s="6">
+      <c r="N88" s="13">
         <f>IF(A88="","",TODAY())</f>
         <v/>
       </c>
@@ -3647,7 +3634,7 @@
         <v/>
       </c>
       <c r="M89" s="4" t="n"/>
-      <c r="N89" s="6">
+      <c r="N89" s="13">
         <f>IF(A89="","",TODAY())</f>
         <v/>
       </c>
@@ -3669,7 +3656,7 @@
         <v/>
       </c>
       <c r="M90" s="4" t="n"/>
-      <c r="N90" s="6">
+      <c r="N90" s="13">
         <f>IF(A90="","",TODAY())</f>
         <v/>
       </c>
@@ -3691,7 +3678,7 @@
         <v/>
       </c>
       <c r="M91" s="4" t="n"/>
-      <c r="N91" s="6">
+      <c r="N91" s="13">
         <f>IF(A91="","",TODAY())</f>
         <v/>
       </c>
@@ -3713,7 +3700,7 @@
         <v/>
       </c>
       <c r="M92" s="4" t="n"/>
-      <c r="N92" s="6">
+      <c r="N92" s="13">
         <f>IF(A92="","",TODAY())</f>
         <v/>
       </c>
@@ -3735,7 +3722,7 @@
         <v/>
       </c>
       <c r="M93" s="4" t="n"/>
-      <c r="N93" s="6">
+      <c r="N93" s="13">
         <f>IF(A93="","",TODAY())</f>
         <v/>
       </c>
@@ -3757,7 +3744,7 @@
         <v/>
       </c>
       <c r="M94" s="4" t="n"/>
-      <c r="N94" s="6">
+      <c r="N94" s="13">
         <f>IF(A94="","",TODAY())</f>
         <v/>
       </c>
@@ -3779,7 +3766,7 @@
         <v/>
       </c>
       <c r="M95" s="4" t="n"/>
-      <c r="N95" s="6">
+      <c r="N95" s="13">
         <f>IF(A95="","",TODAY())</f>
         <v/>
       </c>
@@ -3801,7 +3788,7 @@
         <v/>
       </c>
       <c r="M96" s="4" t="n"/>
-      <c r="N96" s="6">
+      <c r="N96" s="13">
         <f>IF(A96="","",TODAY())</f>
         <v/>
       </c>
@@ -3823,7 +3810,7 @@
         <v/>
       </c>
       <c r="M97" s="4" t="n"/>
-      <c r="N97" s="6">
+      <c r="N97" s="13">
         <f>IF(A97="","",TODAY())</f>
         <v/>
       </c>
@@ -3845,7 +3832,7 @@
         <v/>
       </c>
       <c r="M98" s="4" t="n"/>
-      <c r="N98" s="6">
+      <c r="N98" s="13">
         <f>IF(A98="","",TODAY())</f>
         <v/>
       </c>
@@ -3867,7 +3854,7 @@
         <v/>
       </c>
       <c r="M99" s="4" t="n"/>
-      <c r="N99" s="6">
+      <c r="N99" s="13">
         <f>IF(A99="","",TODAY())</f>
         <v/>
       </c>
@@ -3889,7 +3876,7 @@
         <v/>
       </c>
       <c r="M100" s="4" t="n"/>
-      <c r="N100" s="6">
+      <c r="N100" s="13">
         <f>IF(A100="","",TODAY())</f>
         <v/>
       </c>
@@ -3911,7 +3898,7 @@
         <v/>
       </c>
       <c r="M101" s="4" t="n"/>
-      <c r="N101" s="6">
+      <c r="N101" s="13">
         <f>IF(A101="","",TODAY())</f>
         <v/>
       </c>
@@ -3933,7 +3920,7 @@
         <v/>
       </c>
       <c r="M102" s="4" t="n"/>
-      <c r="N102" s="6">
+      <c r="N102" s="13">
         <f>IF(A102="","",TODAY())</f>
         <v/>
       </c>
@@ -3955,7 +3942,7 @@
         <v/>
       </c>
       <c r="M103" s="4" t="n"/>
-      <c r="N103" s="6">
+      <c r="N103" s="13">
         <f>IF(A103="","",TODAY())</f>
         <v/>
       </c>
@@ -3977,7 +3964,7 @@
         <v/>
       </c>
       <c r="M104" s="4" t="n"/>
-      <c r="N104" s="6">
+      <c r="N104" s="13">
         <f>IF(A104="","",TODAY())</f>
         <v/>
       </c>
@@ -3999,7 +3986,7 @@
         <v/>
       </c>
       <c r="M105" s="4" t="n"/>
-      <c r="N105" s="6">
+      <c r="N105" s="13">
         <f>IF(A105="","",TODAY())</f>
         <v/>
       </c>
@@ -4021,7 +4008,7 @@
         <v/>
       </c>
       <c r="M106" s="4" t="n"/>
-      <c r="N106" s="6">
+      <c r="N106" s="13">
         <f>IF(A106="","",TODAY())</f>
         <v/>
       </c>
@@ -4043,7 +4030,7 @@
         <v/>
       </c>
       <c r="M107" s="4" t="n"/>
-      <c r="N107" s="6">
+      <c r="N107" s="13">
         <f>IF(A107="","",TODAY())</f>
         <v/>
       </c>
@@ -4065,7 +4052,7 @@
         <v/>
       </c>
       <c r="M108" s="4" t="n"/>
-      <c r="N108" s="6">
+      <c r="N108" s="13">
         <f>IF(A108="","",TODAY())</f>
         <v/>
       </c>
@@ -4087,7 +4074,7 @@
         <v/>
       </c>
       <c r="M109" s="4" t="n"/>
-      <c r="N109" s="6">
+      <c r="N109" s="13">
         <f>IF(A109="","",TODAY())</f>
         <v/>
       </c>
@@ -4109,7 +4096,7 @@
         <v/>
       </c>
       <c r="M110" s="4" t="n"/>
-      <c r="N110" s="6">
+      <c r="N110" s="13">
         <f>IF(A110="","",TODAY())</f>
         <v/>
       </c>
@@ -4131,7 +4118,7 @@
         <v/>
       </c>
       <c r="M111" s="4" t="n"/>
-      <c r="N111" s="6">
+      <c r="N111" s="13">
         <f>IF(A111="","",TODAY())</f>
         <v/>
       </c>
@@ -4153,7 +4140,7 @@
         <v/>
       </c>
       <c r="M112" s="4" t="n"/>
-      <c r="N112" s="6">
+      <c r="N112" s="13">
         <f>IF(A112="","",TODAY())</f>
         <v/>
       </c>
@@ -4175,7 +4162,7 @@
         <v/>
       </c>
       <c r="M113" s="4" t="n"/>
-      <c r="N113" s="6">
+      <c r="N113" s="13">
         <f>IF(A113="","",TODAY())</f>
         <v/>
       </c>
@@ -4197,7 +4184,7 @@
         <v/>
       </c>
       <c r="M114" s="4" t="n"/>
-      <c r="N114" s="6">
+      <c r="N114" s="13">
         <f>IF(A114="","",TODAY())</f>
         <v/>
       </c>
@@ -4219,7 +4206,7 @@
         <v/>
       </c>
       <c r="M115" s="4" t="n"/>
-      <c r="N115" s="6">
+      <c r="N115" s="13">
         <f>IF(A115="","",TODAY())</f>
         <v/>
       </c>
@@ -4241,7 +4228,7 @@
         <v/>
       </c>
       <c r="M116" s="4" t="n"/>
-      <c r="N116" s="6">
+      <c r="N116" s="13">
         <f>IF(A116="","",TODAY())</f>
         <v/>
       </c>
@@ -4263,7 +4250,7 @@
         <v/>
       </c>
       <c r="M117" s="4" t="n"/>
-      <c r="N117" s="6">
+      <c r="N117" s="13">
         <f>IF(A117="","",TODAY())</f>
         <v/>
       </c>
@@ -4285,7 +4272,7 @@
         <v/>
       </c>
       <c r="M118" s="4" t="n"/>
-      <c r="N118" s="6">
+      <c r="N118" s="13">
         <f>IF(A118="","",TODAY())</f>
         <v/>
       </c>
@@ -4307,7 +4294,7 @@
         <v/>
       </c>
       <c r="M119" s="4" t="n"/>
-      <c r="N119" s="6">
+      <c r="N119" s="13">
         <f>IF(A119="","",TODAY())</f>
         <v/>
       </c>
@@ -4329,7 +4316,7 @@
         <v/>
       </c>
       <c r="M120" s="4" t="n"/>
-      <c r="N120" s="6">
+      <c r="N120" s="13">
         <f>IF(A120="","",TODAY())</f>
         <v/>
       </c>
@@ -4351,7 +4338,7 @@
         <v/>
       </c>
       <c r="M121" s="4" t="n"/>
-      <c r="N121" s="6">
+      <c r="N121" s="13">
         <f>IF(A121="","",TODAY())</f>
         <v/>
       </c>
@@ -4373,7 +4360,7 @@
         <v/>
       </c>
       <c r="M122" s="4" t="n"/>
-      <c r="N122" s="6">
+      <c r="N122" s="13">
         <f>IF(A122="","",TODAY())</f>
         <v/>
       </c>
@@ -4395,7 +4382,7 @@
         <v/>
       </c>
       <c r="M123" s="4" t="n"/>
-      <c r="N123" s="6">
+      <c r="N123" s="13">
         <f>IF(A123="","",TODAY())</f>
         <v/>
       </c>
@@ -4417,7 +4404,7 @@
         <v/>
       </c>
       <c r="M124" s="4" t="n"/>
-      <c r="N124" s="6">
+      <c r="N124" s="13">
         <f>IF(A124="","",TODAY())</f>
         <v/>
       </c>
@@ -4439,7 +4426,7 @@
         <v/>
       </c>
       <c r="M125" s="4" t="n"/>
-      <c r="N125" s="6">
+      <c r="N125" s="13">
         <f>IF(A125="","",TODAY())</f>
         <v/>
       </c>
@@ -4461,7 +4448,7 @@
         <v/>
       </c>
       <c r="M126" s="4" t="n"/>
-      <c r="N126" s="6">
+      <c r="N126" s="13">
         <f>IF(A126="","",TODAY())</f>
         <v/>
       </c>
@@ -4483,7 +4470,7 @@
         <v/>
       </c>
       <c r="M127" s="4" t="n"/>
-      <c r="N127" s="6">
+      <c r="N127" s="13">
         <f>IF(A127="","",TODAY())</f>
         <v/>
       </c>
@@ -4505,7 +4492,7 @@
         <v/>
       </c>
       <c r="M128" s="4" t="n"/>
-      <c r="N128" s="6">
+      <c r="N128" s="13">
         <f>IF(A128="","",TODAY())</f>
         <v/>
       </c>
@@ -4527,7 +4514,7 @@
         <v/>
       </c>
       <c r="M129" s="4" t="n"/>
-      <c r="N129" s="6">
+      <c r="N129" s="13">
         <f>IF(A129="","",TODAY())</f>
         <v/>
       </c>
@@ -4549,7 +4536,7 @@
         <v/>
       </c>
       <c r="M130" s="4" t="n"/>
-      <c r="N130" s="6">
+      <c r="N130" s="13">
         <f>IF(A130="","",TODAY())</f>
         <v/>
       </c>
@@ -4571,7 +4558,7 @@
         <v/>
       </c>
       <c r="M131" s="4" t="n"/>
-      <c r="N131" s="6">
+      <c r="N131" s="13">
         <f>IF(A131="","",TODAY())</f>
         <v/>
       </c>
@@ -4593,7 +4580,7 @@
         <v/>
       </c>
       <c r="M132" s="4" t="n"/>
-      <c r="N132" s="6">
+      <c r="N132" s="13">
         <f>IF(A132="","",TODAY())</f>
         <v/>
       </c>
@@ -4615,7 +4602,7 @@
         <v/>
       </c>
       <c r="M133" s="4" t="n"/>
-      <c r="N133" s="6">
+      <c r="N133" s="13">
         <f>IF(A133="","",TODAY())</f>
         <v/>
       </c>
@@ -4637,7 +4624,7 @@
         <v/>
       </c>
       <c r="M134" s="4" t="n"/>
-      <c r="N134" s="6">
+      <c r="N134" s="13">
         <f>IF(A134="","",TODAY())</f>
         <v/>
       </c>
@@ -4659,7 +4646,7 @@
         <v/>
       </c>
       <c r="M135" s="4" t="n"/>
-      <c r="N135" s="6">
+      <c r="N135" s="13">
         <f>IF(A135="","",TODAY())</f>
         <v/>
       </c>
@@ -4681,7 +4668,7 @@
         <v/>
       </c>
       <c r="M136" s="4" t="n"/>
-      <c r="N136" s="6">
+      <c r="N136" s="13">
         <f>IF(A136="","",TODAY())</f>
         <v/>
       </c>
@@ -4703,7 +4690,7 @@
         <v/>
       </c>
       <c r="M137" s="4" t="n"/>
-      <c r="N137" s="6">
+      <c r="N137" s="13">
         <f>IF(A137="","",TODAY())</f>
         <v/>
       </c>
@@ -4725,7 +4712,7 @@
         <v/>
       </c>
       <c r="M138" s="4" t="n"/>
-      <c r="N138" s="6">
+      <c r="N138" s="13">
         <f>IF(A138="","",TODAY())</f>
         <v/>
       </c>
@@ -4747,7 +4734,7 @@
         <v/>
       </c>
       <c r="M139" s="4" t="n"/>
-      <c r="N139" s="6">
+      <c r="N139" s="13">
         <f>IF(A139="","",TODAY())</f>
         <v/>
       </c>
@@ -4769,7 +4756,7 @@
         <v/>
       </c>
       <c r="M140" s="4" t="n"/>
-      <c r="N140" s="6">
+      <c r="N140" s="13">
         <f>IF(A140="","",TODAY())</f>
         <v/>
       </c>
@@ -4791,7 +4778,7 @@
         <v/>
       </c>
       <c r="M141" s="4" t="n"/>
-      <c r="N141" s="6">
+      <c r="N141" s="13">
         <f>IF(A141="","",TODAY())</f>
         <v/>
       </c>
@@ -4813,7 +4800,7 @@
         <v/>
       </c>
       <c r="M142" s="4" t="n"/>
-      <c r="N142" s="6">
+      <c r="N142" s="13">
         <f>IF(A142="","",TODAY())</f>
         <v/>
       </c>
@@ -4835,7 +4822,7 @@
         <v/>
       </c>
       <c r="M143" s="4" t="n"/>
-      <c r="N143" s="6">
+      <c r="N143" s="13">
         <f>IF(A143="","",TODAY())</f>
         <v/>
       </c>
@@ -4857,7 +4844,7 @@
         <v/>
       </c>
       <c r="M144" s="4" t="n"/>
-      <c r="N144" s="6">
+      <c r="N144" s="13">
         <f>IF(A144="","",TODAY())</f>
         <v/>
       </c>
@@ -4879,7 +4866,7 @@
         <v/>
       </c>
       <c r="M145" s="4" t="n"/>
-      <c r="N145" s="6">
+      <c r="N145" s="13">
         <f>IF(A145="","",TODAY())</f>
         <v/>
       </c>
@@ -4901,7 +4888,7 @@
         <v/>
       </c>
       <c r="M146" s="4" t="n"/>
-      <c r="N146" s="6">
+      <c r="N146" s="13">
         <f>IF(A146="","",TODAY())</f>
         <v/>
       </c>
@@ -4923,7 +4910,7 @@
         <v/>
       </c>
       <c r="M147" s="4" t="n"/>
-      <c r="N147" s="6">
+      <c r="N147" s="13">
         <f>IF(A147="","",TODAY())</f>
         <v/>
       </c>
@@ -4945,7 +4932,7 @@
         <v/>
       </c>
       <c r="M148" s="4" t="n"/>
-      <c r="N148" s="6">
+      <c r="N148" s="13">
         <f>IF(A148="","",TODAY())</f>
         <v/>
       </c>
@@ -4967,7 +4954,7 @@
         <v/>
       </c>
       <c r="M149" s="4" t="n"/>
-      <c r="N149" s="6">
+      <c r="N149" s="13">
         <f>IF(A149="","",TODAY())</f>
         <v/>
       </c>
@@ -4989,7 +4976,7 @@
         <v/>
       </c>
       <c r="M150" s="4" t="n"/>
-      <c r="N150" s="6">
+      <c r="N150" s="13">
         <f>IF(A150="","",TODAY())</f>
         <v/>
       </c>
@@ -5011,7 +4998,7 @@
         <v/>
       </c>
       <c r="M151" s="4" t="n"/>
-      <c r="N151" s="6">
+      <c r="N151" s="13">
         <f>IF(A151="","",TODAY())</f>
         <v/>
       </c>
@@ -5033,7 +5020,7 @@
         <v/>
       </c>
       <c r="M152" s="4" t="n"/>
-      <c r="N152" s="6">
+      <c r="N152" s="13">
         <f>IF(A152="","",TODAY())</f>
         <v/>
       </c>
@@ -5055,7 +5042,7 @@
         <v/>
       </c>
       <c r="M153" s="4" t="n"/>
-      <c r="N153" s="6">
+      <c r="N153" s="13">
         <f>IF(A153="","",TODAY())</f>
         <v/>
       </c>
@@ -5077,7 +5064,7 @@
         <v/>
       </c>
       <c r="M154" s="4" t="n"/>
-      <c r="N154" s="6">
+      <c r="N154" s="13">
         <f>IF(A154="","",TODAY())</f>
         <v/>
       </c>
@@ -5099,7 +5086,7 @@
         <v/>
       </c>
       <c r="M155" s="4" t="n"/>
-      <c r="N155" s="6">
+      <c r="N155" s="13">
         <f>IF(A155="","",TODAY())</f>
         <v/>
       </c>
@@ -5121,7 +5108,7 @@
         <v/>
       </c>
       <c r="M156" s="4" t="n"/>
-      <c r="N156" s="6">
+      <c r="N156" s="13">
         <f>IF(A156="","",TODAY())</f>
         <v/>
       </c>
@@ -5143,7 +5130,7 @@
         <v/>
       </c>
       <c r="M157" s="4" t="n"/>
-      <c r="N157" s="6">
+      <c r="N157" s="13">
         <f>IF(A157="","",TODAY())</f>
         <v/>
       </c>
@@ -5165,7 +5152,7 @@
         <v/>
       </c>
       <c r="M158" s="4" t="n"/>
-      <c r="N158" s="6">
+      <c r="N158" s="13">
         <f>IF(A158="","",TODAY())</f>
         <v/>
       </c>
@@ -5187,7 +5174,7 @@
         <v/>
       </c>
       <c r="M159" s="4" t="n"/>
-      <c r="N159" s="6">
+      <c r="N159" s="13">
         <f>IF(A159="","",TODAY())</f>
         <v/>
       </c>
@@ -5209,7 +5196,7 @@
         <v/>
       </c>
       <c r="M160" s="4" t="n"/>
-      <c r="N160" s="6">
+      <c r="N160" s="13">
         <f>IF(A160="","",TODAY())</f>
         <v/>
       </c>
@@ -5231,7 +5218,7 @@
         <v/>
       </c>
       <c r="M161" s="4" t="n"/>
-      <c r="N161" s="6">
+      <c r="N161" s="13">
         <f>IF(A161="","",TODAY())</f>
         <v/>
       </c>
@@ -5253,7 +5240,7 @@
         <v/>
       </c>
       <c r="M162" s="4" t="n"/>
-      <c r="N162" s="6">
+      <c r="N162" s="13">
         <f>IF(A162="","",TODAY())</f>
         <v/>
       </c>
@@ -5275,7 +5262,7 @@
         <v/>
       </c>
       <c r="M163" s="4" t="n"/>
-      <c r="N163" s="6">
+      <c r="N163" s="13">
         <f>IF(A163="","",TODAY())</f>
         <v/>
       </c>
@@ -5297,7 +5284,7 @@
         <v/>
       </c>
       <c r="M164" s="4" t="n"/>
-      <c r="N164" s="6">
+      <c r="N164" s="13">
         <f>IF(A164="","",TODAY())</f>
         <v/>
       </c>
@@ -5319,7 +5306,7 @@
         <v/>
       </c>
       <c r="M165" s="4" t="n"/>
-      <c r="N165" s="6">
+      <c r="N165" s="13">
         <f>IF(A165="","",TODAY())</f>
         <v/>
       </c>
@@ -5341,7 +5328,7 @@
         <v/>
       </c>
       <c r="M166" s="4" t="n"/>
-      <c r="N166" s="6">
+      <c r="N166" s="13">
         <f>IF(A166="","",TODAY())</f>
         <v/>
       </c>
@@ -5363,7 +5350,7 @@
         <v/>
       </c>
       <c r="M167" s="4" t="n"/>
-      <c r="N167" s="6">
+      <c r="N167" s="13">
         <f>IF(A167="","",TODAY())</f>
         <v/>
       </c>
@@ -5385,7 +5372,7 @@
         <v/>
       </c>
       <c r="M168" s="4" t="n"/>
-      <c r="N168" s="6">
+      <c r="N168" s="13">
         <f>IF(A168="","",TODAY())</f>
         <v/>
       </c>
@@ -5407,7 +5394,7 @@
         <v/>
       </c>
       <c r="M169" s="4" t="n"/>
-      <c r="N169" s="6">
+      <c r="N169" s="13">
         <f>IF(A169="","",TODAY())</f>
         <v/>
       </c>
@@ -5429,7 +5416,7 @@
         <v/>
       </c>
       <c r="M170" s="4" t="n"/>
-      <c r="N170" s="6">
+      <c r="N170" s="13">
         <f>IF(A170="","",TODAY())</f>
         <v/>
       </c>
@@ -5451,7 +5438,7 @@
         <v/>
       </c>
       <c r="M171" s="4" t="n"/>
-      <c r="N171" s="6">
+      <c r="N171" s="13">
         <f>IF(A171="","",TODAY())</f>
         <v/>
       </c>
@@ -5473,7 +5460,7 @@
         <v/>
       </c>
       <c r="M172" s="4" t="n"/>
-      <c r="N172" s="6">
+      <c r="N172" s="13">
         <f>IF(A172="","",TODAY())</f>
         <v/>
       </c>
@@ -5495,7 +5482,7 @@
         <v/>
       </c>
       <c r="M173" s="4" t="n"/>
-      <c r="N173" s="6">
+      <c r="N173" s="13">
         <f>IF(A173="","",TODAY())</f>
         <v/>
       </c>
@@ -5517,7 +5504,7 @@
         <v/>
       </c>
       <c r="M174" s="4" t="n"/>
-      <c r="N174" s="6">
+      <c r="N174" s="13">
         <f>IF(A174="","",TODAY())</f>
         <v/>
       </c>
@@ -5539,7 +5526,7 @@
         <v/>
       </c>
       <c r="M175" s="4" t="n"/>
-      <c r="N175" s="6">
+      <c r="N175" s="13">
         <f>IF(A175="","",TODAY())</f>
         <v/>
       </c>
@@ -5561,7 +5548,7 @@
         <v/>
       </c>
       <c r="M176" s="4" t="n"/>
-      <c r="N176" s="6">
+      <c r="N176" s="13">
         <f>IF(A176="","",TODAY())</f>
         <v/>
       </c>
@@ -5583,7 +5570,7 @@
         <v/>
       </c>
       <c r="M177" s="4" t="n"/>
-      <c r="N177" s="6">
+      <c r="N177" s="13">
         <f>IF(A177="","",TODAY())</f>
         <v/>
       </c>
@@ -5605,7 +5592,7 @@
         <v/>
       </c>
       <c r="M178" s="4" t="n"/>
-      <c r="N178" s="6">
+      <c r="N178" s="13">
         <f>IF(A178="","",TODAY())</f>
         <v/>
       </c>
@@ -5627,7 +5614,7 @@
         <v/>
       </c>
       <c r="M179" s="4" t="n"/>
-      <c r="N179" s="6">
+      <c r="N179" s="13">
         <f>IF(A179="","",TODAY())</f>
         <v/>
       </c>
@@ -5649,7 +5636,7 @@
         <v/>
       </c>
       <c r="M180" s="4" t="n"/>
-      <c r="N180" s="6">
+      <c r="N180" s="13">
         <f>IF(A180="","",TODAY())</f>
         <v/>
       </c>
@@ -5671,7 +5658,7 @@
         <v/>
       </c>
       <c r="M181" s="4" t="n"/>
-      <c r="N181" s="6">
+      <c r="N181" s="13">
         <f>IF(A181="","",TODAY())</f>
         <v/>
       </c>
@@ -5693,7 +5680,7 @@
         <v/>
       </c>
       <c r="M182" s="4" t="n"/>
-      <c r="N182" s="6">
+      <c r="N182" s="13">
         <f>IF(A182="","",TODAY())</f>
         <v/>
       </c>
@@ -5715,7 +5702,7 @@
         <v/>
       </c>
       <c r="M183" s="4" t="n"/>
-      <c r="N183" s="6">
+      <c r="N183" s="13">
         <f>IF(A183="","",TODAY())</f>
         <v/>
       </c>
@@ -5737,7 +5724,7 @@
         <v/>
       </c>
       <c r="M184" s="4" t="n"/>
-      <c r="N184" s="6">
+      <c r="N184" s="13">
         <f>IF(A184="","",TODAY())</f>
         <v/>
       </c>
@@ -5759,7 +5746,7 @@
         <v/>
       </c>
       <c r="M185" s="4" t="n"/>
-      <c r="N185" s="6">
+      <c r="N185" s="13">
         <f>IF(A185="","",TODAY())</f>
         <v/>
       </c>
@@ -5781,7 +5768,7 @@
         <v/>
       </c>
       <c r="M186" s="4" t="n"/>
-      <c r="N186" s="6">
+      <c r="N186" s="13">
         <f>IF(A186="","",TODAY())</f>
         <v/>
       </c>
@@ -5803,7 +5790,7 @@
         <v/>
       </c>
       <c r="M187" s="4" t="n"/>
-      <c r="N187" s="6">
+      <c r="N187" s="13">
         <f>IF(A187="","",TODAY())</f>
         <v/>
       </c>
@@ -5825,7 +5812,7 @@
         <v/>
       </c>
       <c r="M188" s="4" t="n"/>
-      <c r="N188" s="6">
+      <c r="N188" s="13">
         <f>IF(A188="","",TODAY())</f>
         <v/>
       </c>
@@ -5847,7 +5834,7 @@
         <v/>
       </c>
       <c r="M189" s="4" t="n"/>
-      <c r="N189" s="6">
+      <c r="N189" s="13">
         <f>IF(A189="","",TODAY())</f>
         <v/>
       </c>
@@ -5869,7 +5856,7 @@
         <v/>
       </c>
       <c r="M190" s="4" t="n"/>
-      <c r="N190" s="6">
+      <c r="N190" s="13">
         <f>IF(A190="","",TODAY())</f>
         <v/>
       </c>
@@ -5891,7 +5878,7 @@
         <v/>
       </c>
       <c r="M191" s="4" t="n"/>
-      <c r="N191" s="6">
+      <c r="N191" s="13">
         <f>IF(A191="","",TODAY())</f>
         <v/>
       </c>
@@ -5913,7 +5900,7 @@
         <v/>
       </c>
       <c r="M192" s="4" t="n"/>
-      <c r="N192" s="6">
+      <c r="N192" s="13">
         <f>IF(A192="","",TODAY())</f>
         <v/>
       </c>
@@ -5935,7 +5922,7 @@
         <v/>
       </c>
       <c r="M193" s="4" t="n"/>
-      <c r="N193" s="6">
+      <c r="N193" s="13">
         <f>IF(A193="","",TODAY())</f>
         <v/>
       </c>
@@ -5957,7 +5944,7 @@
         <v/>
       </c>
       <c r="M194" s="4" t="n"/>
-      <c r="N194" s="6">
+      <c r="N194" s="13">
         <f>IF(A194="","",TODAY())</f>
         <v/>
       </c>
@@ -5979,7 +5966,7 @@
         <v/>
       </c>
       <c r="M195" s="4" t="n"/>
-      <c r="N195" s="6">
+      <c r="N195" s="13">
         <f>IF(A195="","",TODAY())</f>
         <v/>
       </c>
@@ -6001,7 +5988,7 @@
         <v/>
       </c>
       <c r="M196" s="4" t="n"/>
-      <c r="N196" s="6">
+      <c r="N196" s="13">
         <f>IF(A196="","",TODAY())</f>
         <v/>
       </c>
@@ -6023,7 +6010,7 @@
         <v/>
       </c>
       <c r="M197" s="4" t="n"/>
-      <c r="N197" s="6">
+      <c r="N197" s="13">
         <f>IF(A197="","",TODAY())</f>
         <v/>
       </c>
@@ -6045,7 +6032,7 @@
         <v/>
       </c>
       <c r="M198" s="4" t="n"/>
-      <c r="N198" s="6">
+      <c r="N198" s="13">
         <f>IF(A198="","",TODAY())</f>
         <v/>
       </c>
@@ -6067,7 +6054,7 @@
         <v/>
       </c>
       <c r="M199" s="4" t="n"/>
-      <c r="N199" s="6">
+      <c r="N199" s="13">
         <f>IF(A199="","",TODAY())</f>
         <v/>
       </c>
@@ -6089,7 +6076,7 @@
         <v/>
       </c>
       <c r="M200" s="4" t="n"/>
-      <c r="N200" s="6">
+      <c r="N200" s="13">
         <f>IF(A200="","",TODAY())</f>
         <v/>
       </c>
@@ -6111,7 +6098,7 @@
         <v/>
       </c>
       <c r="M201" s="4" t="n"/>
-      <c r="N201" s="6">
+      <c r="N201" s="13">
         <f>IF(A201="","",TODAY())</f>
         <v/>
       </c>
@@ -6133,7 +6120,7 @@
         <v/>
       </c>
       <c r="M202" s="4" t="n"/>
-      <c r="N202" s="6">
+      <c r="N202" s="13">
         <f>IF(A202="","",TODAY())</f>
         <v/>
       </c>
@@ -6155,7 +6142,7 @@
         <v/>
       </c>
       <c r="M203" s="4" t="n"/>
-      <c r="N203" s="6">
+      <c r="N203" s="13">
         <f>IF(A203="","",TODAY())</f>
         <v/>
       </c>
@@ -6177,7 +6164,7 @@
         <v/>
       </c>
       <c r="M204" s="4" t="n"/>
-      <c r="N204" s="6">
+      <c r="N204" s="13">
         <f>IF(A204="","",TODAY())</f>
         <v/>
       </c>
@@ -6199,7 +6186,7 @@
         <v/>
       </c>
       <c r="M205" s="4" t="n"/>
-      <c r="N205" s="6">
+      <c r="N205" s="13">
         <f>IF(A205="","",TODAY())</f>
         <v/>
       </c>
@@ -6221,7 +6208,7 @@
         <v/>
       </c>
       <c r="M206" s="4" t="n"/>
-      <c r="N206" s="6">
+      <c r="N206" s="13">
         <f>IF(A206="","",TODAY())</f>
         <v/>
       </c>
@@ -6243,7 +6230,7 @@
         <v/>
       </c>
       <c r="M207" s="4" t="n"/>
-      <c r="N207" s="6">
+      <c r="N207" s="13">
         <f>IF(A207="","",TODAY())</f>
         <v/>
       </c>
@@ -6265,7 +6252,7 @@
         <v/>
       </c>
       <c r="M208" s="4" t="n"/>
-      <c r="N208" s="6">
+      <c r="N208" s="13">
         <f>IF(A208="","",TODAY())</f>
         <v/>
       </c>
@@ -6287,7 +6274,7 @@
         <v/>
       </c>
       <c r="M209" s="4" t="n"/>
-      <c r="N209" s="6">
+      <c r="N209" s="13">
         <f>IF(A209="","",TODAY())</f>
         <v/>
       </c>
@@ -6309,7 +6296,7 @@
         <v/>
       </c>
       <c r="M210" s="4" t="n"/>
-      <c r="N210" s="6">
+      <c r="N210" s="13">
         <f>IF(A210="","",TODAY())</f>
         <v/>
       </c>
@@ -6331,7 +6318,7 @@
         <v/>
       </c>
       <c r="M211" s="4" t="n"/>
-      <c r="N211" s="6">
+      <c r="N211" s="13">
         <f>IF(A211="","",TODAY())</f>
         <v/>
       </c>
@@ -6353,7 +6340,7 @@
         <v/>
       </c>
       <c r="M212" s="4" t="n"/>
-      <c r="N212" s="6">
+      <c r="N212" s="13">
         <f>IF(A212="","",TODAY())</f>
         <v/>
       </c>
@@ -6375,7 +6362,7 @@
         <v/>
       </c>
       <c r="M213" s="4" t="n"/>
-      <c r="N213" s="6">
+      <c r="N213" s="13">
         <f>IF(A213="","",TODAY())</f>
         <v/>
       </c>
@@ -6397,7 +6384,7 @@
         <v/>
       </c>
       <c r="M214" s="4" t="n"/>
-      <c r="N214" s="6">
+      <c r="N214" s="13">
         <f>IF(A214="","",TODAY())</f>
         <v/>
       </c>
@@ -6419,7 +6406,7 @@
         <v/>
       </c>
       <c r="M215" s="4" t="n"/>
-      <c r="N215" s="6">
+      <c r="N215" s="13">
         <f>IF(A215="","",TODAY())</f>
         <v/>
       </c>
@@ -6441,7 +6428,7 @@
         <v/>
       </c>
       <c r="M216" s="4" t="n"/>
-      <c r="N216" s="6">
+      <c r="N216" s="13">
         <f>IF(A216="","",TODAY())</f>
         <v/>
       </c>
@@ -6463,7 +6450,7 @@
         <v/>
       </c>
       <c r="M217" s="4" t="n"/>
-      <c r="N217" s="6">
+      <c r="N217" s="13">
         <f>IF(A217="","",TODAY())</f>
         <v/>
       </c>
@@ -6485,7 +6472,7 @@
         <v/>
       </c>
       <c r="M218" s="4" t="n"/>
-      <c r="N218" s="6">
+      <c r="N218" s="13">
         <f>IF(A218="","",TODAY())</f>
         <v/>
       </c>
@@ -6507,7 +6494,7 @@
         <v/>
       </c>
       <c r="M219" s="4" t="n"/>
-      <c r="N219" s="6">
+      <c r="N219" s="13">
         <f>IF(A219="","",TODAY())</f>
         <v/>
       </c>
@@ -6529,7 +6516,7 @@
         <v/>
       </c>
       <c r="M220" s="4" t="n"/>
-      <c r="N220" s="6">
+      <c r="N220" s="13">
         <f>IF(A220="","",TODAY())</f>
         <v/>
       </c>
@@ -6551,7 +6538,7 @@
         <v/>
       </c>
       <c r="M221" s="4" t="n"/>
-      <c r="N221" s="6">
+      <c r="N221" s="13">
         <f>IF(A221="","",TODAY())</f>
         <v/>
       </c>
@@ -6573,7 +6560,7 @@
         <v/>
       </c>
       <c r="M222" s="4" t="n"/>
-      <c r="N222" s="6">
+      <c r="N222" s="13">
         <f>IF(A222="","",TODAY())</f>
         <v/>
       </c>
@@ -6595,7 +6582,7 @@
         <v/>
       </c>
       <c r="M223" s="4" t="n"/>
-      <c r="N223" s="6">
+      <c r="N223" s="13">
         <f>IF(A223="","",TODAY())</f>
         <v/>
       </c>
@@ -6617,7 +6604,7 @@
         <v/>
       </c>
       <c r="M224" s="4" t="n"/>
-      <c r="N224" s="6">
+      <c r="N224" s="13">
         <f>IF(A224="","",TODAY())</f>
         <v/>
       </c>
@@ -6639,7 +6626,7 @@
         <v/>
       </c>
       <c r="M225" s="4" t="n"/>
-      <c r="N225" s="6">
+      <c r="N225" s="13">
         <f>IF(A225="","",TODAY())</f>
         <v/>
       </c>
@@ -6661,7 +6648,7 @@
         <v/>
       </c>
       <c r="M226" s="4" t="n"/>
-      <c r="N226" s="6">
+      <c r="N226" s="13">
         <f>IF(A226="","",TODAY())</f>
         <v/>
       </c>
@@ -6683,7 +6670,7 @@
         <v/>
       </c>
       <c r="M227" s="4" t="n"/>
-      <c r="N227" s="6">
+      <c r="N227" s="13">
         <f>IF(A227="","",TODAY())</f>
         <v/>
       </c>
@@ -6705,7 +6692,7 @@
         <v/>
       </c>
       <c r="M228" s="4" t="n"/>
-      <c r="N228" s="6">
+      <c r="N228" s="13">
         <f>IF(A228="","",TODAY())</f>
         <v/>
       </c>
@@ -6727,7 +6714,7 @@
         <v/>
       </c>
       <c r="M229" s="4" t="n"/>
-      <c r="N229" s="6">
+      <c r="N229" s="13">
         <f>IF(A229="","",TODAY())</f>
         <v/>
       </c>
@@ -6749,7 +6736,7 @@
         <v/>
       </c>
       <c r="M230" s="4" t="n"/>
-      <c r="N230" s="6">
+      <c r="N230" s="13">
         <f>IF(A230="","",TODAY())</f>
         <v/>
       </c>
@@ -6771,7 +6758,7 @@
         <v/>
       </c>
       <c r="M231" s="4" t="n"/>
-      <c r="N231" s="6">
+      <c r="N231" s="13">
         <f>IF(A231="","",TODAY())</f>
         <v/>
       </c>
@@ -6793,7 +6780,7 @@
         <v/>
       </c>
       <c r="M232" s="4" t="n"/>
-      <c r="N232" s="6">
+      <c r="N232" s="13">
         <f>IF(A232="","",TODAY())</f>
         <v/>
       </c>
@@ -6815,7 +6802,7 @@
         <v/>
       </c>
       <c r="M233" s="4" t="n"/>
-      <c r="N233" s="6">
+      <c r="N233" s="13">
         <f>IF(A233="","",TODAY())</f>
         <v/>
       </c>
@@ -6837,7 +6824,7 @@
         <v/>
       </c>
       <c r="M234" s="4" t="n"/>
-      <c r="N234" s="6">
+      <c r="N234" s="13">
         <f>IF(A234="","",TODAY())</f>
         <v/>
       </c>
@@ -6859,7 +6846,7 @@
         <v/>
       </c>
       <c r="M235" s="4" t="n"/>
-      <c r="N235" s="6">
+      <c r="N235" s="13">
         <f>IF(A235="","",TODAY())</f>
         <v/>
       </c>
@@ -6881,7 +6868,7 @@
         <v/>
       </c>
       <c r="M236" s="4" t="n"/>
-      <c r="N236" s="6">
+      <c r="N236" s="13">
         <f>IF(A236="","",TODAY())</f>
         <v/>
       </c>
@@ -6903,7 +6890,7 @@
         <v/>
       </c>
       <c r="M237" s="4" t="n"/>
-      <c r="N237" s="6">
+      <c r="N237" s="13">
         <f>IF(A237="","",TODAY())</f>
         <v/>
       </c>
@@ -6925,7 +6912,7 @@
         <v/>
       </c>
       <c r="M238" s="4" t="n"/>
-      <c r="N238" s="6">
+      <c r="N238" s="13">
         <f>IF(A238="","",TODAY())</f>
         <v/>
       </c>
@@ -6947,7 +6934,7 @@
         <v/>
       </c>
       <c r="M239" s="4" t="n"/>
-      <c r="N239" s="6">
+      <c r="N239" s="13">
         <f>IF(A239="","",TODAY())</f>
         <v/>
       </c>
@@ -6969,7 +6956,7 @@
         <v/>
       </c>
       <c r="M240" s="4" t="n"/>
-      <c r="N240" s="6">
+      <c r="N240" s="13">
         <f>IF(A240="","",TODAY())</f>
         <v/>
       </c>
@@ -6991,7 +6978,7 @@
         <v/>
       </c>
       <c r="M241" s="4" t="n"/>
-      <c r="N241" s="6">
+      <c r="N241" s="13">
         <f>IF(A241="","",TODAY())</f>
         <v/>
       </c>
@@ -7013,7 +7000,7 @@
         <v/>
       </c>
       <c r="M242" s="4" t="n"/>
-      <c r="N242" s="6">
+      <c r="N242" s="13">
         <f>IF(A242="","",TODAY())</f>
         <v/>
       </c>
@@ -7035,7 +7022,7 @@
         <v/>
       </c>
       <c r="M243" s="4" t="n"/>
-      <c r="N243" s="6">
+      <c r="N243" s="13">
         <f>IF(A243="","",TODAY())</f>
         <v/>
       </c>
@@ -7057,7 +7044,7 @@
         <v/>
       </c>
       <c r="M244" s="4" t="n"/>
-      <c r="N244" s="6">
+      <c r="N244" s="13">
         <f>IF(A244="","",TODAY())</f>
         <v/>
       </c>
@@ -7079,7 +7066,7 @@
         <v/>
       </c>
       <c r="M245" s="4" t="n"/>
-      <c r="N245" s="6">
+      <c r="N245" s="13">
         <f>IF(A245="","",TODAY())</f>
         <v/>
       </c>
@@ -7101,7 +7088,7 @@
         <v/>
       </c>
       <c r="M246" s="4" t="n"/>
-      <c r="N246" s="6">
+      <c r="N246" s="13">
         <f>IF(A246="","",TODAY())</f>
         <v/>
       </c>
@@ -7123,7 +7110,7 @@
         <v/>
       </c>
       <c r="M247" s="4" t="n"/>
-      <c r="N247" s="6">
+      <c r="N247" s="13">
         <f>IF(A247="","",TODAY())</f>
         <v/>
       </c>
@@ -7145,7 +7132,7 @@
         <v/>
       </c>
       <c r="M248" s="4" t="n"/>
-      <c r="N248" s="6">
+      <c r="N248" s="13">
         <f>IF(A248="","",TODAY())</f>
         <v/>
       </c>
@@ -7167,7 +7154,7 @@
         <v/>
       </c>
       <c r="M249" s="4" t="n"/>
-      <c r="N249" s="6">
+      <c r="N249" s="13">
         <f>IF(A249="","",TODAY())</f>
         <v/>
       </c>
@@ -7189,7 +7176,7 @@
         <v/>
       </c>
       <c r="M250" s="4" t="n"/>
-      <c r="N250" s="6">
+      <c r="N250" s="13">
         <f>IF(A250="","",TODAY())</f>
         <v/>
       </c>
@@ -7211,7 +7198,7 @@
         <v/>
       </c>
       <c r="M251" s="4" t="n"/>
-      <c r="N251" s="6">
+      <c r="N251" s="13">
         <f>IF(A251="","",TODAY())</f>
         <v/>
       </c>
@@ -7233,7 +7220,7 @@
         <v/>
       </c>
       <c r="M252" s="4" t="n"/>
-      <c r="N252" s="6">
+      <c r="N252" s="13">
         <f>IF(A252="","",TODAY())</f>
         <v/>
       </c>
@@ -7255,7 +7242,7 @@
         <v/>
       </c>
       <c r="M253" s="4" t="n"/>
-      <c r="N253" s="6">
+      <c r="N253" s="13">
         <f>IF(A253="","",TODAY())</f>
         <v/>
       </c>
@@ -7277,7 +7264,7 @@
         <v/>
       </c>
       <c r="M254" s="4" t="n"/>
-      <c r="N254" s="6">
+      <c r="N254" s="13">
         <f>IF(A254="","",TODAY())</f>
         <v/>
       </c>
@@ -7299,7 +7286,7 @@
         <v/>
       </c>
       <c r="M255" s="4" t="n"/>
-      <c r="N255" s="6">
+      <c r="N255" s="13">
         <f>IF(A255="","",TODAY())</f>
         <v/>
       </c>
@@ -7321,7 +7308,7 @@
         <v/>
       </c>
       <c r="M256" s="4" t="n"/>
-      <c r="N256" s="6">
+      <c r="N256" s="13">
         <f>IF(A256="","",TODAY())</f>
         <v/>
       </c>
@@ -7343,7 +7330,7 @@
         <v/>
       </c>
       <c r="M257" s="4" t="n"/>
-      <c r="N257" s="6">
+      <c r="N257" s="13">
         <f>IF(A257="","",TODAY())</f>
         <v/>
       </c>
@@ -7365,7 +7352,7 @@
         <v/>
       </c>
       <c r="M258" s="4" t="n"/>
-      <c r="N258" s="6">
+      <c r="N258" s="13">
         <f>IF(A258="","",TODAY())</f>
         <v/>
       </c>
@@ -7387,7 +7374,7 @@
         <v/>
       </c>
       <c r="M259" s="4" t="n"/>
-      <c r="N259" s="6">
+      <c r="N259" s="13">
         <f>IF(A259="","",TODAY())</f>
         <v/>
       </c>
@@ -7409,7 +7396,7 @@
         <v/>
       </c>
       <c r="M260" s="4" t="n"/>
-      <c r="N260" s="6">
+      <c r="N260" s="13">
         <f>IF(A260="","",TODAY())</f>
         <v/>
       </c>
@@ -7431,7 +7418,7 @@
         <v/>
       </c>
       <c r="M261" s="4" t="n"/>
-      <c r="N261" s="6">
+      <c r="N261" s="13">
         <f>IF(A261="","",TODAY())</f>
         <v/>
       </c>
@@ -7453,7 +7440,7 @@
         <v/>
       </c>
       <c r="M262" s="4" t="n"/>
-      <c r="N262" s="6">
+      <c r="N262" s="13">
         <f>IF(A262="","",TODAY())</f>
         <v/>
       </c>
@@ -7475,7 +7462,7 @@
         <v/>
       </c>
       <c r="M263" s="4" t="n"/>
-      <c r="N263" s="6">
+      <c r="N263" s="13">
         <f>IF(A263="","",TODAY())</f>
         <v/>
       </c>
@@ -7497,7 +7484,7 @@
         <v/>
       </c>
       <c r="M264" s="4" t="n"/>
-      <c r="N264" s="6">
+      <c r="N264" s="13">
         <f>IF(A264="","",TODAY())</f>
         <v/>
       </c>
@@ -7519,7 +7506,7 @@
         <v/>
       </c>
       <c r="M265" s="4" t="n"/>
-      <c r="N265" s="6">
+      <c r="N265" s="13">
         <f>IF(A265="","",TODAY())</f>
         <v/>
       </c>
@@ -7541,7 +7528,7 @@
         <v/>
       </c>
       <c r="M266" s="4" t="n"/>
-      <c r="N266" s="6">
+      <c r="N266" s="13">
         <f>IF(A266="","",TODAY())</f>
         <v/>
       </c>
@@ -7563,7 +7550,7 @@
         <v/>
       </c>
       <c r="M267" s="4" t="n"/>
-      <c r="N267" s="6">
+      <c r="N267" s="13">
         <f>IF(A267="","",TODAY())</f>
         <v/>
       </c>
@@ -7585,7 +7572,7 @@
         <v/>
       </c>
       <c r="M268" s="4" t="n"/>
-      <c r="N268" s="6">
+      <c r="N268" s="13">
         <f>IF(A268="","",TODAY())</f>
         <v/>
       </c>
@@ -7607,7 +7594,7 @@
         <v/>
       </c>
       <c r="M269" s="4" t="n"/>
-      <c r="N269" s="6">
+      <c r="N269" s="13">
         <f>IF(A269="","",TODAY())</f>
         <v/>
       </c>
@@ -7629,7 +7616,7 @@
         <v/>
       </c>
       <c r="M270" s="4" t="n"/>
-      <c r="N270" s="6">
+      <c r="N270" s="13">
         <f>IF(A270="","",TODAY())</f>
         <v/>
       </c>
@@ -7651,7 +7638,7 @@
         <v/>
       </c>
       <c r="M271" s="4" t="n"/>
-      <c r="N271" s="6">
+      <c r="N271" s="13">
         <f>IF(A271="","",TODAY())</f>
         <v/>
       </c>
@@ -7673,7 +7660,7 @@
         <v/>
       </c>
       <c r="M272" s="4" t="n"/>
-      <c r="N272" s="6">
+      <c r="N272" s="13">
         <f>IF(A272="","",TODAY())</f>
         <v/>
       </c>
@@ -7695,7 +7682,7 @@
         <v/>
       </c>
       <c r="M273" s="4" t="n"/>
-      <c r="N273" s="6">
+      <c r="N273" s="13">
         <f>IF(A273="","",TODAY())</f>
         <v/>
       </c>
@@ -7717,7 +7704,7 @@
         <v/>
       </c>
       <c r="M274" s="4" t="n"/>
-      <c r="N274" s="6">
+      <c r="N274" s="13">
         <f>IF(A274="","",TODAY())</f>
         <v/>
       </c>
@@ -7739,7 +7726,7 @@
         <v/>
       </c>
       <c r="M275" s="4" t="n"/>
-      <c r="N275" s="6">
+      <c r="N275" s="13">
         <f>IF(A275="","",TODAY())</f>
         <v/>
       </c>
@@ -7761,7 +7748,7 @@
         <v/>
       </c>
       <c r="M276" s="4" t="n"/>
-      <c r="N276" s="6">
+      <c r="N276" s="13">
         <f>IF(A276="","",TODAY())</f>
         <v/>
       </c>
@@ -7783,7 +7770,7 @@
         <v/>
       </c>
       <c r="M277" s="4" t="n"/>
-      <c r="N277" s="6">
+      <c r="N277" s="13">
         <f>IF(A277="","",TODAY())</f>
         <v/>
       </c>
@@ -7805,7 +7792,7 @@
         <v/>
       </c>
       <c r="M278" s="4" t="n"/>
-      <c r="N278" s="6">
+      <c r="N278" s="13">
         <f>IF(A278="","",TODAY())</f>
         <v/>
       </c>
@@ -7827,7 +7814,7 @@
         <v/>
       </c>
       <c r="M279" s="4" t="n"/>
-      <c r="N279" s="6">
+      <c r="N279" s="13">
         <f>IF(A279="","",TODAY())</f>
         <v/>
       </c>
@@ -7849,7 +7836,7 @@
         <v/>
       </c>
       <c r="M280" s="4" t="n"/>
-      <c r="N280" s="6">
+      <c r="N280" s="13">
         <f>IF(A280="","",TODAY())</f>
         <v/>
       </c>
@@ -7871,7 +7858,7 @@
         <v/>
       </c>
       <c r="M281" s="4" t="n"/>
-      <c r="N281" s="6">
+      <c r="N281" s="13">
         <f>IF(A281="","",TODAY())</f>
         <v/>
       </c>
@@ -7893,7 +7880,7 @@
         <v/>
       </c>
       <c r="M282" s="4" t="n"/>
-      <c r="N282" s="6">
+      <c r="N282" s="13">
         <f>IF(A282="","",TODAY())</f>
         <v/>
       </c>
@@ -7915,7 +7902,7 @@
         <v/>
       </c>
       <c r="M283" s="4" t="n"/>
-      <c r="N283" s="6">
+      <c r="N283" s="13">
         <f>IF(A283="","",TODAY())</f>
         <v/>
       </c>
@@ -7937,7 +7924,7 @@
         <v/>
       </c>
       <c r="M284" s="4" t="n"/>
-      <c r="N284" s="6">
+      <c r="N284" s="13">
         <f>IF(A284="","",TODAY())</f>
         <v/>
       </c>
@@ -7959,7 +7946,7 @@
         <v/>
       </c>
       <c r="M285" s="4" t="n"/>
-      <c r="N285" s="6">
+      <c r="N285" s="13">
         <f>IF(A285="","",TODAY())</f>
         <v/>
       </c>
@@ -7981,7 +7968,7 @@
         <v/>
       </c>
       <c r="M286" s="4" t="n"/>
-      <c r="N286" s="6">
+      <c r="N286" s="13">
         <f>IF(A286="","",TODAY())</f>
         <v/>
       </c>
@@ -8003,7 +7990,7 @@
         <v/>
       </c>
       <c r="M287" s="4" t="n"/>
-      <c r="N287" s="6">
+      <c r="N287" s="13">
         <f>IF(A287="","",TODAY())</f>
         <v/>
       </c>
@@ -8025,7 +8012,7 @@
         <v/>
       </c>
       <c r="M288" s="4" t="n"/>
-      <c r="N288" s="6">
+      <c r="N288" s="13">
         <f>IF(A288="","",TODAY())</f>
         <v/>
       </c>
@@ -8047,7 +8034,7 @@
         <v/>
       </c>
       <c r="M289" s="4" t="n"/>
-      <c r="N289" s="6">
+      <c r="N289" s="13">
         <f>IF(A289="","",TODAY())</f>
         <v/>
       </c>
@@ -8069,7 +8056,7 @@
         <v/>
       </c>
       <c r="M290" s="4" t="n"/>
-      <c r="N290" s="6">
+      <c r="N290" s="13">
         <f>IF(A290="","",TODAY())</f>
         <v/>
       </c>
@@ -8091,7 +8078,7 @@
         <v/>
       </c>
       <c r="M291" s="4" t="n"/>
-      <c r="N291" s="6">
+      <c r="N291" s="13">
         <f>IF(A291="","",TODAY())</f>
         <v/>
       </c>
@@ -8113,7 +8100,7 @@
         <v/>
       </c>
       <c r="M292" s="4" t="n"/>
-      <c r="N292" s="6">
+      <c r="N292" s="13">
         <f>IF(A292="","",TODAY())</f>
         <v/>
       </c>
@@ -8135,7 +8122,7 @@
         <v/>
       </c>
       <c r="M293" s="4" t="n"/>
-      <c r="N293" s="6">
+      <c r="N293" s="13">
         <f>IF(A293="","",TODAY())</f>
         <v/>
       </c>
@@ -8157,7 +8144,7 @@
         <v/>
       </c>
       <c r="M294" s="4" t="n"/>
-      <c r="N294" s="6">
+      <c r="N294" s="13">
         <f>IF(A294="","",TODAY())</f>
         <v/>
       </c>
@@ -8179,7 +8166,7 @@
         <v/>
       </c>
       <c r="M295" s="4" t="n"/>
-      <c r="N295" s="6">
+      <c r="N295" s="13">
         <f>IF(A295="","",TODAY())</f>
         <v/>
       </c>
@@ -8201,7 +8188,7 @@
         <v/>
       </c>
       <c r="M296" s="4" t="n"/>
-      <c r="N296" s="6">
+      <c r="N296" s="13">
         <f>IF(A296="","",TODAY())</f>
         <v/>
       </c>
@@ -8223,7 +8210,7 @@
         <v/>
       </c>
       <c r="M297" s="4" t="n"/>
-      <c r="N297" s="6">
+      <c r="N297" s="13">
         <f>IF(A297="","",TODAY())</f>
         <v/>
       </c>
@@ -8245,7 +8232,7 @@
         <v/>
       </c>
       <c r="M298" s="4" t="n"/>
-      <c r="N298" s="6">
+      <c r="N298" s="13">
         <f>IF(A298="","",TODAY())</f>
         <v/>
       </c>
@@ -8267,7 +8254,7 @@
         <v/>
       </c>
       <c r="M299" s="4" t="n"/>
-      <c r="N299" s="6">
+      <c r="N299" s="13">
         <f>IF(A299="","",TODAY())</f>
         <v/>
       </c>
@@ -8289,7 +8276,7 @@
         <v/>
       </c>
       <c r="M300" s="4" t="n"/>
-      <c r="N300" s="6">
+      <c r="N300" s="13">
         <f>IF(A300="","",TODAY())</f>
         <v/>
       </c>
@@ -8311,7 +8298,7 @@
         <v/>
       </c>
       <c r="M301" s="4" t="n"/>
-      <c r="N301" s="6">
+      <c r="N301" s="13">
         <f>IF(A301="","",TODAY())</f>
         <v/>
       </c>
@@ -8333,7 +8320,7 @@
         <v/>
       </c>
       <c r="M302" s="4" t="n"/>
-      <c r="N302" s="6">
+      <c r="N302" s="13">
         <f>IF(A302="","",TODAY())</f>
         <v/>
       </c>
@@ -8355,7 +8342,7 @@
         <v/>
       </c>
       <c r="M303" s="4" t="n"/>
-      <c r="N303" s="6">
+      <c r="N303" s="13">
         <f>IF(A303="","",TODAY())</f>
         <v/>
       </c>
@@ -8377,7 +8364,7 @@
         <v/>
       </c>
       <c r="M304" s="4" t="n"/>
-      <c r="N304" s="6">
+      <c r="N304" s="13">
         <f>IF(A304="","",TODAY())</f>
         <v/>
       </c>
@@ -8399,7 +8386,7 @@
         <v/>
       </c>
       <c r="M305" s="4" t="n"/>
-      <c r="N305" s="6">
+      <c r="N305" s="13">
         <f>IF(A305="","",TODAY())</f>
         <v/>
       </c>
@@ -8421,7 +8408,7 @@
         <v/>
       </c>
       <c r="M306" s="4" t="n"/>
-      <c r="N306" s="6">
+      <c r="N306" s="13">
         <f>IF(A306="","",TODAY())</f>
         <v/>
       </c>
@@ -8443,7 +8430,7 @@
         <v/>
       </c>
       <c r="M307" s="4" t="n"/>
-      <c r="N307" s="6">
+      <c r="N307" s="13">
         <f>IF(A307="","",TODAY())</f>
         <v/>
       </c>
@@ -8465,7 +8452,7 @@
         <v/>
       </c>
       <c r="M308" s="4" t="n"/>
-      <c r="N308" s="6">
+      <c r="N308" s="13">
         <f>IF(A308="","",TODAY())</f>
         <v/>
       </c>
@@ -8487,7 +8474,7 @@
         <v/>
       </c>
       <c r="M309" s="4" t="n"/>
-      <c r="N309" s="6">
+      <c r="N309" s="13">
         <f>IF(A309="","",TODAY())</f>
         <v/>
       </c>
@@ -8509,7 +8496,7 @@
         <v/>
       </c>
       <c r="M310" s="4" t="n"/>
-      <c r="N310" s="6">
+      <c r="N310" s="13">
         <f>IF(A310="","",TODAY())</f>
         <v/>
       </c>
@@ -8531,7 +8518,7 @@
         <v/>
       </c>
       <c r="M311" s="4" t="n"/>
-      <c r="N311" s="6">
+      <c r="N311" s="13">
         <f>IF(A311="","",TODAY())</f>
         <v/>
       </c>
@@ -8553,7 +8540,7 @@
         <v/>
       </c>
       <c r="M312" s="4" t="n"/>
-      <c r="N312" s="6">
+      <c r="N312" s="13">
         <f>IF(A312="","",TODAY())</f>
         <v/>
       </c>
@@ -8575,7 +8562,7 @@
         <v/>
       </c>
       <c r="M313" s="4" t="n"/>
-      <c r="N313" s="6">
+      <c r="N313" s="13">
         <f>IF(A313="","",TODAY())</f>
         <v/>
       </c>
@@ -8597,7 +8584,7 @@
         <v/>
       </c>
       <c r="M314" s="4" t="n"/>
-      <c r="N314" s="6">
+      <c r="N314" s="13">
         <f>IF(A314="","",TODAY())</f>
         <v/>
       </c>
@@ -8619,7 +8606,7 @@
         <v/>
       </c>
       <c r="M315" s="4" t="n"/>
-      <c r="N315" s="6">
+      <c r="N315" s="13">
         <f>IF(A315="","",TODAY())</f>
         <v/>
       </c>
@@ -8641,7 +8628,7 @@
         <v/>
       </c>
       <c r="M316" s="4" t="n"/>
-      <c r="N316" s="6">
+      <c r="N316" s="13">
         <f>IF(A316="","",TODAY())</f>
         <v/>
       </c>
@@ -8663,7 +8650,7 @@
         <v/>
       </c>
       <c r="M317" s="4" t="n"/>
-      <c r="N317" s="6">
+      <c r="N317" s="13">
         <f>IF(A317="","",TODAY())</f>
         <v/>
       </c>
@@ -8685,7 +8672,7 @@
         <v/>
       </c>
       <c r="M318" s="4" t="n"/>
-      <c r="N318" s="6">
+      <c r="N318" s="13">
         <f>IF(A318="","",TODAY())</f>
         <v/>
       </c>
@@ -8707,7 +8694,7 @@
         <v/>
       </c>
       <c r="M319" s="4" t="n"/>
-      <c r="N319" s="6">
+      <c r="N319" s="13">
         <f>IF(A319="","",TODAY())</f>
         <v/>
       </c>
@@ -8729,7 +8716,7 @@
         <v/>
       </c>
       <c r="M320" s="4" t="n"/>
-      <c r="N320" s="6">
+      <c r="N320" s="13">
         <f>IF(A320="","",TODAY())</f>
         <v/>
       </c>
@@ -8751,7 +8738,7 @@
         <v/>
       </c>
       <c r="M321" s="4" t="n"/>
-      <c r="N321" s="6">
+      <c r="N321" s="13">
         <f>IF(A321="","",TODAY())</f>
         <v/>
       </c>
@@ -8773,7 +8760,7 @@
         <v/>
       </c>
       <c r="M322" s="4" t="n"/>
-      <c r="N322" s="6">
+      <c r="N322" s="13">
         <f>IF(A322="","",TODAY())</f>
         <v/>
       </c>
@@ -8795,7 +8782,7 @@
         <v/>
       </c>
       <c r="M323" s="4" t="n"/>
-      <c r="N323" s="6">
+      <c r="N323" s="13">
         <f>IF(A323="","",TODAY())</f>
         <v/>
       </c>
@@ -8817,7 +8804,7 @@
         <v/>
       </c>
       <c r="M324" s="4" t="n"/>
-      <c r="N324" s="6">
+      <c r="N324" s="13">
         <f>IF(A324="","",TODAY())</f>
         <v/>
       </c>
@@ -8839,7 +8826,7 @@
         <v/>
       </c>
       <c r="M325" s="4" t="n"/>
-      <c r="N325" s="6">
+      <c r="N325" s="13">
         <f>IF(A325="","",TODAY())</f>
         <v/>
       </c>
@@ -8861,7 +8848,7 @@
         <v/>
       </c>
       <c r="M326" s="4" t="n"/>
-      <c r="N326" s="6">
+      <c r="N326" s="13">
         <f>IF(A326="","",TODAY())</f>
         <v/>
       </c>
@@ -8883,7 +8870,7 @@
         <v/>
       </c>
       <c r="M327" s="4" t="n"/>
-      <c r="N327" s="6">
+      <c r="N327" s="13">
         <f>IF(A327="","",TODAY())</f>
         <v/>
       </c>
@@ -8905,7 +8892,7 @@
         <v/>
       </c>
       <c r="M328" s="4" t="n"/>
-      <c r="N328" s="6">
+      <c r="N328" s="13">
         <f>IF(A328="","",TODAY())</f>
         <v/>
       </c>
@@ -8927,7 +8914,7 @@
         <v/>
       </c>
       <c r="M329" s="4" t="n"/>
-      <c r="N329" s="6">
+      <c r="N329" s="13">
         <f>IF(A329="","",TODAY())</f>
         <v/>
       </c>
@@ -8949,7 +8936,7 @@
         <v/>
       </c>
       <c r="M330" s="4" t="n"/>
-      <c r="N330" s="6">
+      <c r="N330" s="13">
         <f>IF(A330="","",TODAY())</f>
         <v/>
       </c>
@@ -8971,7 +8958,7 @@
         <v/>
       </c>
       <c r="M331" s="4" t="n"/>
-      <c r="N331" s="6">
+      <c r="N331" s="13">
         <f>IF(A331="","",TODAY())</f>
         <v/>
       </c>
@@ -8993,7 +8980,7 @@
         <v/>
       </c>
       <c r="M332" s="4" t="n"/>
-      <c r="N332" s="6">
+      <c r="N332" s="13">
         <f>IF(A332="","",TODAY())</f>
         <v/>
       </c>
@@ -9015,7 +9002,7 @@
         <v/>
       </c>
       <c r="M333" s="4" t="n"/>
-      <c r="N333" s="6">
+      <c r="N333" s="13">
         <f>IF(A333="","",TODAY())</f>
         <v/>
       </c>
@@ -9037,7 +9024,7 @@
         <v/>
       </c>
       <c r="M334" s="4" t="n"/>
-      <c r="N334" s="6">
+      <c r="N334" s="13">
         <f>IF(A334="","",TODAY())</f>
         <v/>
       </c>
@@ -9059,7 +9046,7 @@
         <v/>
       </c>
       <c r="M335" s="4" t="n"/>
-      <c r="N335" s="6">
+      <c r="N335" s="13">
         <f>IF(A335="","",TODAY())</f>
         <v/>
       </c>
@@ -9081,7 +9068,7 @@
         <v/>
       </c>
       <c r="M336" s="4" t="n"/>
-      <c r="N336" s="6">
+      <c r="N336" s="13">
         <f>IF(A336="","",TODAY())</f>
         <v/>
       </c>
@@ -9103,7 +9090,7 @@
         <v/>
       </c>
       <c r="M337" s="4" t="n"/>
-      <c r="N337" s="6">
+      <c r="N337" s="13">
         <f>IF(A337="","",TODAY())</f>
         <v/>
       </c>
@@ -9125,7 +9112,7 @@
         <v/>
       </c>
       <c r="M338" s="4" t="n"/>
-      <c r="N338" s="6">
+      <c r="N338" s="13">
         <f>IF(A338="","",TODAY())</f>
         <v/>
       </c>
@@ -9147,7 +9134,7 @@
         <v/>
       </c>
       <c r="M339" s="4" t="n"/>
-      <c r="N339" s="6">
+      <c r="N339" s="13">
         <f>IF(A339="","",TODAY())</f>
         <v/>
       </c>
@@ -9169,7 +9156,7 @@
         <v/>
       </c>
       <c r="M340" s="4" t="n"/>
-      <c r="N340" s="6">
+      <c r="N340" s="13">
         <f>IF(A340="","",TODAY())</f>
         <v/>
       </c>
@@ -9191,7 +9178,7 @@
         <v/>
       </c>
       <c r="M341" s="4" t="n"/>
-      <c r="N341" s="6">
+      <c r="N341" s="13">
         <f>IF(A341="","",TODAY())</f>
         <v/>
       </c>
@@ -9213,7 +9200,7 @@
         <v/>
       </c>
       <c r="M342" s="4" t="n"/>
-      <c r="N342" s="6">
+      <c r="N342" s="13">
         <f>IF(A342="","",TODAY())</f>
         <v/>
       </c>
@@ -9235,7 +9222,7 @@
         <v/>
       </c>
       <c r="M343" s="4" t="n"/>
-      <c r="N343" s="6">
+      <c r="N343" s="13">
         <f>IF(A343="","",TODAY())</f>
         <v/>
       </c>
@@ -9257,7 +9244,7 @@
         <v/>
       </c>
       <c r="M344" s="4" t="n"/>
-      <c r="N344" s="6">
+      <c r="N344" s="13">
         <f>IF(A344="","",TODAY())</f>
         <v/>
       </c>
@@ -9279,7 +9266,7 @@
         <v/>
       </c>
       <c r="M345" s="4" t="n"/>
-      <c r="N345" s="6">
+      <c r="N345" s="13">
         <f>IF(A345="","",TODAY())</f>
         <v/>
       </c>
@@ -9301,7 +9288,7 @@
         <v/>
       </c>
       <c r="M346" s="4" t="n"/>
-      <c r="N346" s="6">
+      <c r="N346" s="13">
         <f>IF(A346="","",TODAY())</f>
         <v/>
       </c>
@@ -9323,7 +9310,7 @@
         <v/>
       </c>
       <c r="M347" s="4" t="n"/>
-      <c r="N347" s="6">
+      <c r="N347" s="13">
         <f>IF(A347="","",TODAY())</f>
         <v/>
       </c>
@@ -9345,7 +9332,7 @@
         <v/>
       </c>
       <c r="M348" s="4" t="n"/>
-      <c r="N348" s="6">
+      <c r="N348" s="13">
         <f>IF(A348="","",TODAY())</f>
         <v/>
       </c>
@@ -9367,7 +9354,7 @@
         <v/>
       </c>
       <c r="M349" s="4" t="n"/>
-      <c r="N349" s="6">
+      <c r="N349" s="13">
         <f>IF(A349="","",TODAY())</f>
         <v/>
       </c>
@@ -9389,7 +9376,7 @@
         <v/>
       </c>
       <c r="M350" s="4" t="n"/>
-      <c r="N350" s="6">
+      <c r="N350" s="13">
         <f>IF(A350="","",TODAY())</f>
         <v/>
       </c>
@@ -9411,7 +9398,7 @@
         <v/>
       </c>
       <c r="M351" s="4" t="n"/>
-      <c r="N351" s="6">
+      <c r="N351" s="13">
         <f>IF(A351="","",TODAY())</f>
         <v/>
       </c>
@@ -9433,7 +9420,7 @@
         <v/>
       </c>
       <c r="M352" s="4" t="n"/>
-      <c r="N352" s="6">
+      <c r="N352" s="13">
         <f>IF(A352="","",TODAY())</f>
         <v/>
       </c>
@@ -9455,7 +9442,7 @@
         <v/>
       </c>
       <c r="M353" s="4" t="n"/>
-      <c r="N353" s="6">
+      <c r="N353" s="13">
         <f>IF(A353="","",TODAY())</f>
         <v/>
       </c>
@@ -9477,7 +9464,7 @@
         <v/>
       </c>
       <c r="M354" s="4" t="n"/>
-      <c r="N354" s="6">
+      <c r="N354" s="13">
         <f>IF(A354="","",TODAY())</f>
         <v/>
       </c>
@@ -9499,7 +9486,7 @@
         <v/>
       </c>
       <c r="M355" s="4" t="n"/>
-      <c r="N355" s="6">
+      <c r="N355" s="13">
         <f>IF(A355="","",TODAY())</f>
         <v/>
       </c>
@@ -9521,7 +9508,7 @@
         <v/>
       </c>
       <c r="M356" s="4" t="n"/>
-      <c r="N356" s="6">
+      <c r="N356" s="13">
         <f>IF(A356="","",TODAY())</f>
         <v/>
       </c>
@@ -9543,7 +9530,7 @@
         <v/>
       </c>
       <c r="M357" s="4" t="n"/>
-      <c r="N357" s="6">
+      <c r="N357" s="13">
         <f>IF(A357="","",TODAY())</f>
         <v/>
       </c>
@@ -9565,7 +9552,7 @@
         <v/>
       </c>
       <c r="M358" s="4" t="n"/>
-      <c r="N358" s="6">
+      <c r="N358" s="13">
         <f>IF(A358="","",TODAY())</f>
         <v/>
       </c>
@@ -9587,7 +9574,7 @@
         <v/>
       </c>
       <c r="M359" s="4" t="n"/>
-      <c r="N359" s="6">
+      <c r="N359" s="13">
         <f>IF(A359="","",TODAY())</f>
         <v/>
       </c>
@@ -9609,7 +9596,7 @@
         <v/>
       </c>
       <c r="M360" s="4" t="n"/>
-      <c r="N360" s="6">
+      <c r="N360" s="13">
         <f>IF(A360="","",TODAY())</f>
         <v/>
       </c>
@@ -9631,7 +9618,7 @@
         <v/>
       </c>
       <c r="M361" s="4" t="n"/>
-      <c r="N361" s="6">
+      <c r="N361" s="13">
         <f>IF(A361="","",TODAY())</f>
         <v/>
       </c>
@@ -9653,7 +9640,7 @@
         <v/>
       </c>
       <c r="M362" s="4" t="n"/>
-      <c r="N362" s="6">
+      <c r="N362" s="13">
         <f>IF(A362="","",TODAY())</f>
         <v/>
       </c>
@@ -9675,7 +9662,7 @@
         <v/>
       </c>
       <c r="M363" s="4" t="n"/>
-      <c r="N363" s="6">
+      <c r="N363" s="13">
         <f>IF(A363="","",TODAY())</f>
         <v/>
       </c>
@@ -9697,7 +9684,7 @@
         <v/>
       </c>
       <c r="M364" s="4" t="n"/>
-      <c r="N364" s="6">
+      <c r="N364" s="13">
         <f>IF(A364="","",TODAY())</f>
         <v/>
       </c>
@@ -9719,7 +9706,7 @@
         <v/>
       </c>
       <c r="M365" s="4" t="n"/>
-      <c r="N365" s="6">
+      <c r="N365" s="13">
         <f>IF(A365="","",TODAY())</f>
         <v/>
       </c>
@@ -9741,7 +9728,7 @@
         <v/>
       </c>
       <c r="M366" s="4" t="n"/>
-      <c r="N366" s="6">
+      <c r="N366" s="13">
         <f>IF(A366="","",TODAY())</f>
         <v/>
       </c>
@@ -9763,7 +9750,7 @@
         <v/>
       </c>
       <c r="M367" s="4" t="n"/>
-      <c r="N367" s="6">
+      <c r="N367" s="13">
         <f>IF(A367="","",TODAY())</f>
         <v/>
       </c>
@@ -9785,7 +9772,7 @@
         <v/>
       </c>
       <c r="M368" s="4" t="n"/>
-      <c r="N368" s="6">
+      <c r="N368" s="13">
         <f>IF(A368="","",TODAY())</f>
         <v/>
       </c>
@@ -9807,7 +9794,7 @@
         <v/>
       </c>
       <c r="M369" s="4" t="n"/>
-      <c r="N369" s="6">
+      <c r="N369" s="13">
         <f>IF(A369="","",TODAY())</f>
         <v/>
       </c>
@@ -9829,7 +9816,7 @@
         <v/>
       </c>
       <c r="M370" s="4" t="n"/>
-      <c r="N370" s="6">
+      <c r="N370" s="13">
         <f>IF(A370="","",TODAY())</f>
         <v/>
       </c>
@@ -9851,7 +9838,7 @@
         <v/>
       </c>
       <c r="M371" s="4" t="n"/>
-      <c r="N371" s="6">
+      <c r="N371" s="13">
         <f>IF(A371="","",TODAY())</f>
         <v/>
       </c>
@@ -9873,7 +9860,7 @@
         <v/>
       </c>
       <c r="M372" s="4" t="n"/>
-      <c r="N372" s="6">
+      <c r="N372" s="13">
         <f>IF(A372="","",TODAY())</f>
         <v/>
       </c>
@@ -9895,7 +9882,7 @@
         <v/>
       </c>
       <c r="M373" s="4" t="n"/>
-      <c r="N373" s="6">
+      <c r="N373" s="13">
         <f>IF(A373="","",TODAY())</f>
         <v/>
       </c>
@@ -9917,7 +9904,7 @@
         <v/>
       </c>
       <c r="M374" s="4" t="n"/>
-      <c r="N374" s="6">
+      <c r="N374" s="13">
         <f>IF(A374="","",TODAY())</f>
         <v/>
       </c>
@@ -9939,7 +9926,7 @@
         <v/>
       </c>
       <c r="M375" s="4" t="n"/>
-      <c r="N375" s="6">
+      <c r="N375" s="13">
         <f>IF(A375="","",TODAY())</f>
         <v/>
       </c>
@@ -9961,7 +9948,7 @@
         <v/>
       </c>
       <c r="M376" s="4" t="n"/>
-      <c r="N376" s="6">
+      <c r="N376" s="13">
         <f>IF(A376="","",TODAY())</f>
         <v/>
       </c>
@@ -9983,7 +9970,7 @@
         <v/>
       </c>
       <c r="M377" s="4" t="n"/>
-      <c r="N377" s="6">
+      <c r="N377" s="13">
         <f>IF(A377="","",TODAY())</f>
         <v/>
       </c>
@@ -10005,7 +9992,7 @@
         <v/>
       </c>
       <c r="M378" s="4" t="n"/>
-      <c r="N378" s="6">
+      <c r="N378" s="13">
         <f>IF(A378="","",TODAY())</f>
         <v/>
       </c>
@@ -10027,7 +10014,7 @@
         <v/>
       </c>
       <c r="M379" s="4" t="n"/>
-      <c r="N379" s="6">
+      <c r="N379" s="13">
         <f>IF(A379="","",TODAY())</f>
         <v/>
       </c>
@@ -10049,7 +10036,7 @@
         <v/>
       </c>
       <c r="M380" s="4" t="n"/>
-      <c r="N380" s="6">
+      <c r="N380" s="13">
         <f>IF(A380="","",TODAY())</f>
         <v/>
       </c>
@@ -10071,7 +10058,7 @@
         <v/>
       </c>
       <c r="M381" s="4" t="n"/>
-      <c r="N381" s="6">
+      <c r="N381" s="13">
         <f>IF(A381="","",TODAY())</f>
         <v/>
       </c>
@@ -10093,7 +10080,7 @@
         <v/>
       </c>
       <c r="M382" s="4" t="n"/>
-      <c r="N382" s="6">
+      <c r="N382" s="13">
         <f>IF(A382="","",TODAY())</f>
         <v/>
       </c>
@@ -10115,7 +10102,7 @@
         <v/>
       </c>
       <c r="M383" s="4" t="n"/>
-      <c r="N383" s="6">
+      <c r="N383" s="13">
         <f>IF(A383="","",TODAY())</f>
         <v/>
       </c>
@@ -10137,7 +10124,7 @@
         <v/>
       </c>
       <c r="M384" s="4" t="n"/>
-      <c r="N384" s="6">
+      <c r="N384" s="13">
         <f>IF(A384="","",TODAY())</f>
         <v/>
       </c>
@@ -10159,7 +10146,7 @@
         <v/>
       </c>
       <c r="M385" s="4" t="n"/>
-      <c r="N385" s="6">
+      <c r="N385" s="13">
         <f>IF(A385="","",TODAY())</f>
         <v/>
       </c>
@@ -10181,7 +10168,7 @@
         <v/>
       </c>
       <c r="M386" s="4" t="n"/>
-      <c r="N386" s="6">
+      <c r="N386" s="13">
         <f>IF(A386="","",TODAY())</f>
         <v/>
       </c>
@@ -10203,7 +10190,7 @@
         <v/>
       </c>
       <c r="M387" s="4" t="n"/>
-      <c r="N387" s="6">
+      <c r="N387" s="13">
         <f>IF(A387="","",TODAY())</f>
         <v/>
       </c>
@@ -10225,7 +10212,7 @@
         <v/>
       </c>
       <c r="M388" s="4" t="n"/>
-      <c r="N388" s="6">
+      <c r="N388" s="13">
         <f>IF(A388="","",TODAY())</f>
         <v/>
       </c>
@@ -10247,7 +10234,7 @@
         <v/>
       </c>
       <c r="M389" s="4" t="n"/>
-      <c r="N389" s="6">
+      <c r="N389" s="13">
         <f>IF(A389="","",TODAY())</f>
         <v/>
       </c>
@@ -10269,7 +10256,7 @@
         <v/>
       </c>
       <c r="M390" s="4" t="n"/>
-      <c r="N390" s="6">
+      <c r="N390" s="13">
         <f>IF(A390="","",TODAY())</f>
         <v/>
       </c>
@@ -10291,7 +10278,7 @@
         <v/>
       </c>
       <c r="M391" s="4" t="n"/>
-      <c r="N391" s="6">
+      <c r="N391" s="13">
         <f>IF(A391="","",TODAY())</f>
         <v/>
       </c>
@@ -10313,7 +10300,7 @@
         <v/>
       </c>
       <c r="M392" s="4" t="n"/>
-      <c r="N392" s="6">
+      <c r="N392" s="13">
         <f>IF(A392="","",TODAY())</f>
         <v/>
       </c>
@@ -10335,7 +10322,7 @@
         <v/>
       </c>
       <c r="M393" s="4" t="n"/>
-      <c r="N393" s="6">
+      <c r="N393" s="13">
         <f>IF(A393="","",TODAY())</f>
         <v/>
       </c>
@@ -10357,7 +10344,7 @@
         <v/>
       </c>
       <c r="M394" s="4" t="n"/>
-      <c r="N394" s="6">
+      <c r="N394" s="13">
         <f>IF(A394="","",TODAY())</f>
         <v/>
       </c>
@@ -10379,7 +10366,7 @@
         <v/>
       </c>
       <c r="M395" s="4" t="n"/>
-      <c r="N395" s="6">
+      <c r="N395" s="13">
         <f>IF(A395="","",TODAY())</f>
         <v/>
       </c>
@@ -10401,7 +10388,7 @@
         <v/>
       </c>
       <c r="M396" s="4" t="n"/>
-      <c r="N396" s="6">
+      <c r="N396" s="13">
         <f>IF(A396="","",TODAY())</f>
         <v/>
       </c>
@@ -10423,7 +10410,7 @@
         <v/>
       </c>
       <c r="M397" s="4" t="n"/>
-      <c r="N397" s="6">
+      <c r="N397" s="13">
         <f>IF(A397="","",TODAY())</f>
         <v/>
       </c>
@@ -10445,7 +10432,7 @@
         <v/>
       </c>
       <c r="M398" s="4" t="n"/>
-      <c r="N398" s="6">
+      <c r="N398" s="13">
         <f>IF(A398="","",TODAY())</f>
         <v/>
       </c>
@@ -10467,7 +10454,7 @@
         <v/>
       </c>
       <c r="M399" s="4" t="n"/>
-      <c r="N399" s="6">
+      <c r="N399" s="13">
         <f>IF(A399="","",TODAY())</f>
         <v/>
       </c>
@@ -10489,7 +10476,7 @@
         <v/>
       </c>
       <c r="M400" s="4" t="n"/>
-      <c r="N400" s="6">
+      <c r="N400" s="13">
         <f>IF(A400="","",TODAY())</f>
         <v/>
       </c>
@@ -10511,7 +10498,7 @@
         <v/>
       </c>
       <c r="M401" s="4" t="n"/>
-      <c r="N401" s="6">
+      <c r="N401" s="13">
         <f>IF(A401="","",TODAY())</f>
         <v/>
       </c>
@@ -10533,7 +10520,7 @@
         <v/>
       </c>
       <c r="M402" s="4" t="n"/>
-      <c r="N402" s="6">
+      <c r="N402" s="13">
         <f>IF(A402="","",TODAY())</f>
         <v/>
       </c>
@@ -10555,7 +10542,7 @@
         <v/>
       </c>
       <c r="M403" s="4" t="n"/>
-      <c r="N403" s="6">
+      <c r="N403" s="13">
         <f>IF(A403="","",TODAY())</f>
         <v/>
       </c>
@@ -10577,7 +10564,7 @@
         <v/>
       </c>
       <c r="M404" s="4" t="n"/>
-      <c r="N404" s="6">
+      <c r="N404" s="13">
         <f>IF(A404="","",TODAY())</f>
         <v/>
       </c>
@@ -10599,7 +10586,7 @@
         <v/>
       </c>
       <c r="M405" s="4" t="n"/>
-      <c r="N405" s="6">
+      <c r="N405" s="13">
         <f>IF(A405="","",TODAY())</f>
         <v/>
       </c>
@@ -10621,7 +10608,7 @@
         <v/>
       </c>
       <c r="M406" s="4" t="n"/>
-      <c r="N406" s="6">
+      <c r="N406" s="13">
         <f>IF(A406="","",TODAY())</f>
         <v/>
       </c>
@@ -10643,7 +10630,7 @@
         <v/>
       </c>
       <c r="M407" s="4" t="n"/>
-      <c r="N407" s="6">
+      <c r="N407" s="13">
         <f>IF(A407="","",TODAY())</f>
         <v/>
       </c>
@@ -10665,7 +10652,7 @@
         <v/>
       </c>
       <c r="M408" s="4" t="n"/>
-      <c r="N408" s="6">
+      <c r="N408" s="13">
         <f>IF(A408="","",TODAY())</f>
         <v/>
       </c>
@@ -10687,7 +10674,7 @@
         <v/>
       </c>
       <c r="M409" s="4" t="n"/>
-      <c r="N409" s="6">
+      <c r="N409" s="13">
         <f>IF(A409="","",TODAY())</f>
         <v/>
       </c>
@@ -10709,7 +10696,7 @@
         <v/>
       </c>
       <c r="M410" s="4" t="n"/>
-      <c r="N410" s="6">
+      <c r="N410" s="13">
         <f>IF(A410="","",TODAY())</f>
         <v/>
       </c>
@@ -10731,7 +10718,7 @@
         <v/>
       </c>
       <c r="M411" s="4" t="n"/>
-      <c r="N411" s="6">
+      <c r="N411" s="13">
         <f>IF(A411="","",TODAY())</f>
         <v/>
       </c>
@@ -10753,7 +10740,7 @@
         <v/>
       </c>
       <c r="M412" s="4" t="n"/>
-      <c r="N412" s="6">
+      <c r="N412" s="13">
         <f>IF(A412="","",TODAY())</f>
         <v/>
       </c>
@@ -10775,7 +10762,7 @@
         <v/>
       </c>
       <c r="M413" s="4" t="n"/>
-      <c r="N413" s="6">
+      <c r="N413" s="13">
         <f>IF(A413="","",TODAY())</f>
         <v/>
       </c>
@@ -10797,7 +10784,7 @@
         <v/>
       </c>
       <c r="M414" s="4" t="n"/>
-      <c r="N414" s="6">
+      <c r="N414" s="13">
         <f>IF(A414="","",TODAY())</f>
         <v/>
       </c>
@@ -10819,7 +10806,7 @@
         <v/>
       </c>
       <c r="M415" s="4" t="n"/>
-      <c r="N415" s="6">
+      <c r="N415" s="13">
         <f>IF(A415="","",TODAY())</f>
         <v/>
       </c>
@@ -10841,7 +10828,7 @@
         <v/>
       </c>
       <c r="M416" s="4" t="n"/>
-      <c r="N416" s="6">
+      <c r="N416" s="13">
         <f>IF(A416="","",TODAY())</f>
         <v/>
       </c>
@@ -10863,7 +10850,7 @@
         <v/>
       </c>
       <c r="M417" s="4" t="n"/>
-      <c r="N417" s="6">
+      <c r="N417" s="13">
         <f>IF(A417="","",TODAY())</f>
         <v/>
       </c>
@@ -10885,7 +10872,7 @@
         <v/>
       </c>
       <c r="M418" s="4" t="n"/>
-      <c r="N418" s="6">
+      <c r="N418" s="13">
         <f>IF(A418="","",TODAY())</f>
         <v/>
       </c>
@@ -10907,7 +10894,7 @@
         <v/>
       </c>
       <c r="M419" s="4" t="n"/>
-      <c r="N419" s="6">
+      <c r="N419" s="13">
         <f>IF(A419="","",TODAY())</f>
         <v/>
       </c>
@@ -10929,7 +10916,7 @@
         <v/>
       </c>
       <c r="M420" s="4" t="n"/>
-      <c r="N420" s="6">
+      <c r="N420" s="13">
         <f>IF(A420="","",TODAY())</f>
         <v/>
       </c>
@@ -10951,7 +10938,7 @@
         <v/>
       </c>
       <c r="M421" s="4" t="n"/>
-      <c r="N421" s="6">
+      <c r="N421" s="13">
         <f>IF(A421="","",TODAY())</f>
         <v/>
       </c>
@@ -10973,7 +10960,7 @@
         <v/>
       </c>
       <c r="M422" s="4" t="n"/>
-      <c r="N422" s="6">
+      <c r="N422" s="13">
         <f>IF(A422="","",TODAY())</f>
         <v/>
       </c>
@@ -10995,7 +10982,7 @@
         <v/>
       </c>
       <c r="M423" s="4" t="n"/>
-      <c r="N423" s="6">
+      <c r="N423" s="13">
         <f>IF(A423="","",TODAY())</f>
         <v/>
       </c>
@@ -11017,7 +11004,7 @@
         <v/>
       </c>
       <c r="M424" s="4" t="n"/>
-      <c r="N424" s="6">
+      <c r="N424" s="13">
         <f>IF(A424="","",TODAY())</f>
         <v/>
       </c>
@@ -11039,7 +11026,7 @@
         <v/>
       </c>
       <c r="M425" s="4" t="n"/>
-      <c r="N425" s="6">
+      <c r="N425" s="13">
         <f>IF(A425="","",TODAY())</f>
         <v/>
       </c>
@@ -11061,7 +11048,7 @@
         <v/>
       </c>
       <c r="M426" s="4" t="n"/>
-      <c r="N426" s="6">
+      <c r="N426" s="13">
         <f>IF(A426="","",TODAY())</f>
         <v/>
       </c>
@@ -11083,7 +11070,7 @@
         <v/>
       </c>
       <c r="M427" s="4" t="n"/>
-      <c r="N427" s="6">
+      <c r="N427" s="13">
         <f>IF(A427="","",TODAY())</f>
         <v/>
       </c>
@@ -11105,7 +11092,7 @@
         <v/>
       </c>
       <c r="M428" s="4" t="n"/>
-      <c r="N428" s="6">
+      <c r="N428" s="13">
         <f>IF(A428="","",TODAY())</f>
         <v/>
       </c>
@@ -11127,7 +11114,7 @@
         <v/>
       </c>
       <c r="M429" s="4" t="n"/>
-      <c r="N429" s="6">
+      <c r="N429" s="13">
         <f>IF(A429="","",TODAY())</f>
         <v/>
       </c>
@@ -11149,7 +11136,7 @@
         <v/>
       </c>
       <c r="M430" s="4" t="n"/>
-      <c r="N430" s="6">
+      <c r="N430" s="13">
         <f>IF(A430="","",TODAY())</f>
         <v/>
       </c>
@@ -11171,7 +11158,7 @@
         <v/>
       </c>
       <c r="M431" s="4" t="n"/>
-      <c r="N431" s="6">
+      <c r="N431" s="13">
         <f>IF(A431="","",TODAY())</f>
         <v/>
       </c>
@@ -11193,7 +11180,7 @@
         <v/>
       </c>
       <c r="M432" s="4" t="n"/>
-      <c r="N432" s="6">
+      <c r="N432" s="13">
         <f>IF(A432="","",TODAY())</f>
         <v/>
       </c>
@@ -11215,7 +11202,7 @@
         <v/>
       </c>
       <c r="M433" s="4" t="n"/>
-      <c r="N433" s="6">
+      <c r="N433" s="13">
         <f>IF(A433="","",TODAY())</f>
         <v/>
       </c>
@@ -11237,7 +11224,7 @@
         <v/>
       </c>
       <c r="M434" s="4" t="n"/>
-      <c r="N434" s="6">
+      <c r="N434" s="13">
         <f>IF(A434="","",TODAY())</f>
         <v/>
       </c>
@@ -11259,7 +11246,7 @@
         <v/>
       </c>
       <c r="M435" s="4" t="n"/>
-      <c r="N435" s="6">
+      <c r="N435" s="13">
         <f>IF(A435="","",TODAY())</f>
         <v/>
       </c>
@@ -11281,7 +11268,7 @@
         <v/>
       </c>
       <c r="M436" s="4" t="n"/>
-      <c r="N436" s="6">
+      <c r="N436" s="13">
         <f>IF(A436="","",TODAY())</f>
         <v/>
       </c>
@@ -11303,7 +11290,7 @@
         <v/>
       </c>
       <c r="M437" s="4" t="n"/>
-      <c r="N437" s="6">
+      <c r="N437" s="13">
         <f>IF(A437="","",TODAY())</f>
         <v/>
       </c>
@@ -11325,7 +11312,7 @@
         <v/>
       </c>
       <c r="M438" s="4" t="n"/>
-      <c r="N438" s="6">
+      <c r="N438" s="13">
         <f>IF(A438="","",TODAY())</f>
         <v/>
       </c>
@@ -11347,7 +11334,7 @@
         <v/>
       </c>
       <c r="M439" s="4" t="n"/>
-      <c r="N439" s="6">
+      <c r="N439" s="13">
         <f>IF(A439="","",TODAY())</f>
         <v/>
       </c>
@@ -11369,7 +11356,7 @@
         <v/>
       </c>
       <c r="M440" s="4" t="n"/>
-      <c r="N440" s="6">
+      <c r="N440" s="13">
         <f>IF(A440="","",TODAY())</f>
         <v/>
       </c>
@@ -11391,7 +11378,7 @@
         <v/>
       </c>
       <c r="M441" s="4" t="n"/>
-      <c r="N441" s="6">
+      <c r="N441" s="13">
         <f>IF(A441="","",TODAY())</f>
         <v/>
       </c>
@@ -11413,7 +11400,7 @@
         <v/>
       </c>
       <c r="M442" s="4" t="n"/>
-      <c r="N442" s="6">
+      <c r="N442" s="13">
         <f>IF(A442="","",TODAY())</f>
         <v/>
       </c>
@@ -11435,7 +11422,7 @@
         <v/>
       </c>
       <c r="M443" s="4" t="n"/>
-      <c r="N443" s="6">
+      <c r="N443" s="13">
         <f>IF(A443="","",TODAY())</f>
         <v/>
       </c>
@@ -11457,7 +11444,7 @@
         <v/>
       </c>
       <c r="M444" s="4" t="n"/>
-      <c r="N444" s="6">
+      <c r="N444" s="13">
         <f>IF(A444="","",TODAY())</f>
         <v/>
       </c>
@@ -11479,7 +11466,7 @@
         <v/>
       </c>
       <c r="M445" s="4" t="n"/>
-      <c r="N445" s="6">
+      <c r="N445" s="13">
         <f>IF(A445="","",TODAY())</f>
         <v/>
       </c>
@@ -11501,7 +11488,7 @@
         <v/>
       </c>
       <c r="M446" s="4" t="n"/>
-      <c r="N446" s="6">
+      <c r="N446" s="13">
         <f>IF(A446="","",TODAY())</f>
         <v/>
       </c>
@@ -11523,7 +11510,7 @@
         <v/>
       </c>
       <c r="M447" s="4" t="n"/>
-      <c r="N447" s="6">
+      <c r="N447" s="13">
         <f>IF(A447="","",TODAY())</f>
         <v/>
       </c>
@@ -11545,7 +11532,7 @@
         <v/>
       </c>
       <c r="M448" s="4" t="n"/>
-      <c r="N448" s="6">
+      <c r="N448" s="13">
         <f>IF(A448="","",TODAY())</f>
         <v/>
       </c>
@@ -11567,7 +11554,7 @@
         <v/>
       </c>
       <c r="M449" s="4" t="n"/>
-      <c r="N449" s="6">
+      <c r="N449" s="13">
         <f>IF(A449="","",TODAY())</f>
         <v/>
       </c>
@@ -11589,7 +11576,7 @@
         <v/>
       </c>
       <c r="M450" s="4" t="n"/>
-      <c r="N450" s="6">
+      <c r="N450" s="13">
         <f>IF(A450="","",TODAY())</f>
         <v/>
       </c>
@@ -11611,7 +11598,7 @@
         <v/>
       </c>
       <c r="M451" s="4" t="n"/>
-      <c r="N451" s="6">
+      <c r="N451" s="13">
         <f>IF(A451="","",TODAY())</f>
         <v/>
       </c>
@@ -11633,7 +11620,7 @@
         <v/>
       </c>
       <c r="M452" s="4" t="n"/>
-      <c r="N452" s="6">
+      <c r="N452" s="13">
         <f>IF(A452="","",TODAY())</f>
         <v/>
       </c>
@@ -11655,7 +11642,7 @@
         <v/>
       </c>
       <c r="M453" s="4" t="n"/>
-      <c r="N453" s="6">
+      <c r="N453" s="13">
         <f>IF(A453="","",TODAY())</f>
         <v/>
       </c>
@@ -11677,7 +11664,7 @@
         <v/>
       </c>
       <c r="M454" s="4" t="n"/>
-      <c r="N454" s="6">
+      <c r="N454" s="13">
         <f>IF(A454="","",TODAY())</f>
         <v/>
       </c>
@@ -11699,7 +11686,7 @@
         <v/>
       </c>
       <c r="M455" s="4" t="n"/>
-      <c r="N455" s="6">
+      <c r="N455" s="13">
         <f>IF(A455="","",TODAY())</f>
         <v/>
       </c>
@@ -11721,7 +11708,7 @@
         <v/>
       </c>
       <c r="M456" s="4" t="n"/>
-      <c r="N456" s="6">
+      <c r="N456" s="13">
         <f>IF(A456="","",TODAY())</f>
         <v/>
       </c>
@@ -11743,7 +11730,7 @@
         <v/>
       </c>
       <c r="M457" s="4" t="n"/>
-      <c r="N457" s="6">
+      <c r="N457" s="13">
         <f>IF(A457="","",TODAY())</f>
         <v/>
       </c>
@@ -11765,7 +11752,7 @@
         <v/>
       </c>
       <c r="M458" s="4" t="n"/>
-      <c r="N458" s="6">
+      <c r="N458" s="13">
         <f>IF(A458="","",TODAY())</f>
         <v/>
       </c>
@@ -11787,7 +11774,7 @@
         <v/>
       </c>
       <c r="M459" s="4" t="n"/>
-      <c r="N459" s="6">
+      <c r="N459" s="13">
         <f>IF(A459="","",TODAY())</f>
         <v/>
       </c>
@@ -11809,7 +11796,7 @@
         <v/>
       </c>
       <c r="M460" s="4" t="n"/>
-      <c r="N460" s="6">
+      <c r="N460" s="13">
         <f>IF(A460="","",TODAY())</f>
         <v/>
       </c>
@@ -11831,7 +11818,7 @@
         <v/>
       </c>
       <c r="M461" s="4" t="n"/>
-      <c r="N461" s="6">
+      <c r="N461" s="13">
         <f>IF(A461="","",TODAY())</f>
         <v/>
       </c>
@@ -11853,7 +11840,7 @@
         <v/>
       </c>
       <c r="M462" s="4" t="n"/>
-      <c r="N462" s="6">
+      <c r="N462" s="13">
         <f>IF(A462="","",TODAY())</f>
         <v/>
       </c>
@@ -11875,7 +11862,7 @@
         <v/>
       </c>
       <c r="M463" s="4" t="n"/>
-      <c r="N463" s="6">
+      <c r="N463" s="13">
         <f>IF(A463="","",TODAY())</f>
         <v/>
       </c>
@@ -11897,7 +11884,7 @@
         <v/>
       </c>
       <c r="M464" s="4" t="n"/>
-      <c r="N464" s="6">
+      <c r="N464" s="13">
         <f>IF(A464="","",TODAY())</f>
         <v/>
       </c>
@@ -11919,7 +11906,7 @@
         <v/>
       </c>
       <c r="M465" s="4" t="n"/>
-      <c r="N465" s="6">
+      <c r="N465" s="13">
         <f>IF(A465="","",TODAY())</f>
         <v/>
       </c>
@@ -11941,7 +11928,7 @@
         <v/>
       </c>
       <c r="M466" s="4" t="n"/>
-      <c r="N466" s="6">
+      <c r="N466" s="13">
         <f>IF(A466="","",TODAY())</f>
         <v/>
       </c>
@@ -11963,7 +11950,7 @@
         <v/>
       </c>
       <c r="M467" s="4" t="n"/>
-      <c r="N467" s="6">
+      <c r="N467" s="13">
         <f>IF(A467="","",TODAY())</f>
         <v/>
       </c>
@@ -11985,7 +11972,7 @@
         <v/>
       </c>
       <c r="M468" s="4" t="n"/>
-      <c r="N468" s="6">
+      <c r="N468" s="13">
         <f>IF(A468="","",TODAY())</f>
         <v/>
       </c>
@@ -12007,7 +11994,7 @@
         <v/>
       </c>
       <c r="M469" s="4" t="n"/>
-      <c r="N469" s="6">
+      <c r="N469" s="13">
         <f>IF(A469="","",TODAY())</f>
         <v/>
       </c>
@@ -12029,7 +12016,7 @@
         <v/>
       </c>
       <c r="M470" s="4" t="n"/>
-      <c r="N470" s="6">
+      <c r="N470" s="13">
         <f>IF(A470="","",TODAY())</f>
         <v/>
       </c>
@@ -12051,7 +12038,7 @@
         <v/>
       </c>
       <c r="M471" s="4" t="n"/>
-      <c r="N471" s="6">
+      <c r="N471" s="13">
         <f>IF(A471="","",TODAY())</f>
         <v/>
       </c>
@@ -12073,7 +12060,7 @@
         <v/>
       </c>
       <c r="M472" s="4" t="n"/>
-      <c r="N472" s="6">
+      <c r="N472" s="13">
         <f>IF(A472="","",TODAY())</f>
         <v/>
       </c>
@@ -12095,7 +12082,7 @@
         <v/>
       </c>
       <c r="M473" s="4" t="n"/>
-      <c r="N473" s="6">
+      <c r="N473" s="13">
         <f>IF(A473="","",TODAY())</f>
         <v/>
       </c>
@@ -12117,7 +12104,7 @@
         <v/>
       </c>
       <c r="M474" s="4" t="n"/>
-      <c r="N474" s="6">
+      <c r="N474" s="13">
         <f>IF(A474="","",TODAY())</f>
         <v/>
       </c>
@@ -12139,7 +12126,7 @@
         <v/>
       </c>
       <c r="M475" s="4" t="n"/>
-      <c r="N475" s="6">
+      <c r="N475" s="13">
         <f>IF(A475="","",TODAY())</f>
         <v/>
       </c>
@@ -12161,7 +12148,7 @@
         <v/>
       </c>
       <c r="M476" s="4" t="n"/>
-      <c r="N476" s="6">
+      <c r="N476" s="13">
         <f>IF(A476="","",TODAY())</f>
         <v/>
       </c>
@@ -12183,7 +12170,7 @@
         <v/>
       </c>
       <c r="M477" s="4" t="n"/>
-      <c r="N477" s="6">
+      <c r="N477" s="13">
         <f>IF(A477="","",TODAY())</f>
         <v/>
       </c>
@@ -12205,7 +12192,7 @@
         <v/>
       </c>
       <c r="M478" s="4" t="n"/>
-      <c r="N478" s="6">
+      <c r="N478" s="13">
         <f>IF(A478="","",TODAY())</f>
         <v/>
       </c>
@@ -12227,7 +12214,7 @@
         <v/>
       </c>
       <c r="M479" s="4" t="n"/>
-      <c r="N479" s="6">
+      <c r="N479" s="13">
         <f>IF(A479="","",TODAY())</f>
         <v/>
       </c>
@@ -12249,7 +12236,7 @@
         <v/>
       </c>
       <c r="M480" s="4" t="n"/>
-      <c r="N480" s="6">
+      <c r="N480" s="13">
         <f>IF(A480="","",TODAY())</f>
         <v/>
       </c>
@@ -12271,7 +12258,7 @@
         <v/>
       </c>
       <c r="M481" s="4" t="n"/>
-      <c r="N481" s="6">
+      <c r="N481" s="13">
         <f>IF(A481="","",TODAY())</f>
         <v/>
       </c>
@@ -12293,7 +12280,7 @@
         <v/>
       </c>
       <c r="M482" s="4" t="n"/>
-      <c r="N482" s="6">
+      <c r="N482" s="13">
         <f>IF(A482="","",TODAY())</f>
         <v/>
       </c>
@@ -12315,7 +12302,7 @@
         <v/>
       </c>
       <c r="M483" s="4" t="n"/>
-      <c r="N483" s="6">
+      <c r="N483" s="13">
         <f>IF(A483="","",TODAY())</f>
         <v/>
       </c>
@@ -12337,7 +12324,7 @@
         <v/>
       </c>
       <c r="M484" s="4" t="n"/>
-      <c r="N484" s="6">
+      <c r="N484" s="13">
         <f>IF(A484="","",TODAY())</f>
         <v/>
       </c>
@@ -12359,7 +12346,7 @@
         <v/>
       </c>
       <c r="M485" s="4" t="n"/>
-      <c r="N485" s="6">
+      <c r="N485" s="13">
         <f>IF(A485="","",TODAY())</f>
         <v/>
       </c>
@@ -12381,7 +12368,7 @@
         <v/>
       </c>
       <c r="M486" s="4" t="n"/>
-      <c r="N486" s="6">
+      <c r="N486" s="13">
         <f>IF(A486="","",TODAY())</f>
         <v/>
       </c>
@@ -12403,7 +12390,7 @@
         <v/>
       </c>
       <c r="M487" s="4" t="n"/>
-      <c r="N487" s="6">
+      <c r="N487" s="13">
         <f>IF(A487="","",TODAY())</f>
         <v/>
       </c>
@@ -12425,7 +12412,7 @@
         <v/>
       </c>
       <c r="M488" s="4" t="n"/>
-      <c r="N488" s="6">
+      <c r="N488" s="13">
         <f>IF(A488="","",TODAY())</f>
         <v/>
       </c>
@@ -12447,7 +12434,7 @@
         <v/>
       </c>
       <c r="M489" s="4" t="n"/>
-      <c r="N489" s="6">
+      <c r="N489" s="13">
         <f>IF(A489="","",TODAY())</f>
         <v/>
       </c>
@@ -12469,7 +12456,7 @@
         <v/>
       </c>
       <c r="M490" s="4" t="n"/>
-      <c r="N490" s="6">
+      <c r="N490" s="13">
         <f>IF(A490="","",TODAY())</f>
         <v/>
       </c>
@@ -12491,7 +12478,7 @@
         <v/>
       </c>
       <c r="M491" s="4" t="n"/>
-      <c r="N491" s="6">
+      <c r="N491" s="13">
         <f>IF(A491="","",TODAY())</f>
         <v/>
       </c>
@@ -12513,7 +12500,7 @@
         <v/>
       </c>
       <c r="M492" s="4" t="n"/>
-      <c r="N492" s="6">
+      <c r="N492" s="13">
         <f>IF(A492="","",TODAY())</f>
         <v/>
       </c>
@@ -12535,7 +12522,7 @@
         <v/>
       </c>
       <c r="M493" s="4" t="n"/>
-      <c r="N493" s="6">
+      <c r="N493" s="13">
         <f>IF(A493="","",TODAY())</f>
         <v/>
       </c>
@@ -12557,7 +12544,7 @@
         <v/>
       </c>
       <c r="M494" s="4" t="n"/>
-      <c r="N494" s="6">
+      <c r="N494" s="13">
         <f>IF(A494="","",TODAY())</f>
         <v/>
       </c>
@@ -12579,7 +12566,7 @@
         <v/>
       </c>
       <c r="M495" s="4" t="n"/>
-      <c r="N495" s="6">
+      <c r="N495" s="13">
         <f>IF(A495="","",TODAY())</f>
         <v/>
       </c>
@@ -12601,7 +12588,7 @@
         <v/>
       </c>
       <c r="M496" s="4" t="n"/>
-      <c r="N496" s="6">
+      <c r="N496" s="13">
         <f>IF(A496="","",TODAY())</f>
         <v/>
       </c>
@@ -12623,7 +12610,7 @@
         <v/>
       </c>
       <c r="M497" s="4" t="n"/>
-      <c r="N497" s="6">
+      <c r="N497" s="13">
         <f>IF(A497="","",TODAY())</f>
         <v/>
       </c>
@@ -12645,7 +12632,7 @@
         <v/>
       </c>
       <c r="M498" s="4" t="n"/>
-      <c r="N498" s="6">
+      <c r="N498" s="13">
         <f>IF(A498="","",TODAY())</f>
         <v/>
       </c>
@@ -12667,7 +12654,7 @@
         <v/>
       </c>
       <c r="M499" s="4" t="n"/>
-      <c r="N499" s="6">
+      <c r="N499" s="13">
         <f>IF(A499="","",TODAY())</f>
         <v/>
       </c>
@@ -12689,7 +12676,7 @@
         <v/>
       </c>
       <c r="M500" s="4" t="n"/>
-      <c r="N500" s="6">
+      <c r="N500" s="13">
         <f>IF(A500="","",TODAY())</f>
         <v/>
       </c>
@@ -13175,7 +13162,7 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="D8" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"1 квартал")</f>
@@ -13190,7 +13177,7 @@
         <v/>
       </c>
       <c r="G8" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="H8" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"2 квартал")</f>
@@ -13205,7 +13192,7 @@
         <v/>
       </c>
       <c r="K8" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="L8" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"3 квартал")</f>
@@ -13220,7 +13207,7 @@
         <v/>
       </c>
       <c r="O8" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="P8" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A8,Сделки!$B:$B,"4 квартал")</f>
@@ -13247,7 +13234,7 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="D9" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"1 квартал")</f>
@@ -13262,7 +13249,7 @@
         <v/>
       </c>
       <c r="G9" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="H9" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"2 квартал")</f>
@@ -13277,7 +13264,7 @@
         <v/>
       </c>
       <c r="K9" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="L9" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"3 квартал")</f>
@@ -13292,7 +13279,7 @@
         <v/>
       </c>
       <c r="O9" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="P9" s="5">
         <f>SUMIFS(Сделки!$H:$H,Сделки!$D:$D,$A9,Сделки!$B:$B,"4 квартал")</f>
@@ -13456,7 +13443,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -13465,7 +13452,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 60 000 000, квартальный 15 000 000</t>
+          <t>Ориентировочно 5 000 000 на квартал из расчета 60 000 000 в год</t>
         </is>
       </c>
     </row>
@@ -13481,7 +13468,7 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -13490,7 +13477,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 50 000 000, квартальный 12 500 000</t>
+          <t>Ориентировочно 4 000 000 на квартал из расчета 50 000 000 в год</t>
         </is>
       </c>
     </row>
@@ -14162,7 +14149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14409,11 +14396,11 @@
         </is>
       </c>
       <c r="M6" s="5" t="n">
-        <v>15000000</v>
+        <v>5000000</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 60 000 000, квартальный 15 000 000</t>
+          <t>Ориентировочно 5 000 000 на квартал из расчета 60 000 000 в год</t>
         </is>
       </c>
     </row>
@@ -14439,11 +14426,11 @@
         </is>
       </c>
       <c r="M7" s="5" t="n">
-        <v>12500000</v>
+        <v>4000000</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Годовой план 50 000 000, квартальный 12 500 000</t>
+          <t>Ориентировочно 4 000 000 на квартал из расчета 50 000 000 в год</t>
         </is>
       </c>
     </row>
@@ -14494,13 +14481,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <autoFilter ref="A1:N20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14677,6 +14657,5 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add quarterly dashboard breakdown
Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sales_plan_company_filled.xlsx
+++ b/sales_plan_company_filled.xlsx
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,7 @@
       <b val="1"/>
       <sz val="16"/>
     </font>
+    <font/>
   </fonts>
   <fills count="6">
     <fill>
@@ -80,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -102,11 +103,12 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -141,6 +143,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14494,15 +14516,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14644,8 +14669,390 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Разбивка по кварталам</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Квартал</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>План</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Прогноз</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Факт</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Выполнение факта</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Покрытие прогнозом</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Сделок всего</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Обсуждение/риски</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>1 квартал</t>
+        </is>
+      </c>
+      <c r="B15" s="17">
+        <f>SUM(Справочники!$M$2:$M$7)</f>
+        <v/>
+      </c>
+      <c r="C15" s="17">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="D15" s="17">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="E15" s="18">
+        <f>IFERROR(D15/B15,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="18">
+        <f>IFERROR(C15/B15,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2,Сделки!$F:$F,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="H15" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Завершена")</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$B:$B,$A15,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Бюджет под риском")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>2 квартал</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>SUM(Справочники!$M$2:$M$7)</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="D16" s="17">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="E16" s="18">
+        <f>IFERROR(D16/B16,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="18">
+        <f>IFERROR(C16/B16,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2,Сделки!$F:$F,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="H16" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Завершена")</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$B:$B,$A16,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Бюджет под риском")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>3 квартал</t>
+        </is>
+      </c>
+      <c r="B17" s="17">
+        <f>SUM(Справочники!$M$2:$M$7)</f>
+        <v/>
+      </c>
+      <c r="C17" s="17">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="D17" s="17">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>IFERROR(D17/B17,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="18">
+        <f>IFERROR(C17/B17,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2,Сделки!$F:$F,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="H17" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Завершена")</f>
+        <v/>
+      </c>
+      <c r="I17" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$B:$B,$A17,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Бюджет под риском")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>4 квартал</t>
+        </is>
+      </c>
+      <c r="B18" s="17">
+        <f>SUM(Справочники!$M$2:$M$7)</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
+        <f>SUMIFS(Сделки!$H:$H,Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="D18" s="17">
+        <f>SUMIFS(Сделки!$I:$I,Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2)</f>
+        <v/>
+      </c>
+      <c r="E18" s="18">
+        <f>IFERROR(D18/B18,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="18">
+        <f>IFERROR(C18/B18,0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2,Сделки!$F:$F,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="H18" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Завершена")</f>
+        <v/>
+      </c>
+      <c r="I18" s="17">
+        <f>COUNTIFS(Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Обсуждение")+COUNTIFS(Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Потенциал")+COUNTIFS(Сделки!$B:$B,$A18,Сделки!$A:$A,$C$2,Сделки!$J:$J,"Бюджет под риском")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="B19" s="20">
+        <f>SUM(B15:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="20">
+        <f>SUM(C15:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="20">
+        <f>SUM(D15:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>IFERROR(D19/B19,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="21">
+        <f>IFERROR(C19/B19,0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="20">
+        <f>SUM(G15:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="20">
+        <f>SUM(H15:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="20">
+        <f>SUM(I15:I18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="15" t="n"/>
+      <c r="I22" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="n"/>
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="15" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="15" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="n"/>
+      <c r="G27" s="15" t="n"/>
+      <c r="H27" s="15" t="n"/>
+      <c r="I27" s="15" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="15" t="n"/>
+      <c r="H28" s="15" t="n"/>
+      <c r="I28" s="15" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="15" t="n"/>
+      <c r="I29" s="15" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="n"/>
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="n"/>
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="15" t="n"/>
+      <c r="I30" s="15" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A12:I12"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="2">

</xml_diff>